<commit_message>
Doplniť pohľadávky Štefana Nagya Bača a dlžníka YQ House
Šesť položiek pre Štefana Nagya Bača s dátumami splatnosti, štvrtý
dlžník YQ House, odstránený vzorový riadok a pridaný súhrn po dlžníkoch.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L5Qg2mKXdzeFPu6vSu8w6V
</commit_message>
<xml_diff>
--- a/supis_dlhov.xlsx
+++ b/supis_dlhov.xlsx
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="62">
   <si>
     <t xml:space="preserve">Súpis pohľadávok a výpočet úroku z omeškania</t>
   </si>
@@ -108,7 +108,7 @@
     <t xml:space="preserve">Vypočítané: 10 % × 3 / 12 = 2,5 % za štvrťrok.</t>
   </si>
   <si>
-    <t xml:space="preserve">Legenda: žlté bunky s modrým písmom vyplňte (dlžník, titul, istina, dátum, úročiť, stav, poznámka). Biele bunky sú vzorce – neprepisujte ich. Riadok 14 je PRÍKLAD formátu – prepíšte alebo vymažte.</t>
+    <t xml:space="preserve">Legenda: žlté bunky s modrým písmom vyplňte (dlžník, titul, istina, dátum, úročiť, stav, poznámka). Biele bunky sú vzorce – neprepisujte ich. Riadky 11–16 ukazujú formát vyplnenia (dátum DD.MM.RRRR, suma v €).</t>
   </si>
   <si>
     <t xml:space="preserve">Metóda: za každé ukončené 3-mesačné obdobie od dátumu splatnosti sa úrok pripočíta k istine (zložené úročenie). Za nedokončené bežné obdobie sa počíta jednoduchý úrok z kapitalizovanej istiny pomerne podľa dní (rok = 365 dní). Pri „Úročiť = nie“ sa úrok nepočíta a dlžná suma = istina.</t>
@@ -156,18 +156,39 @@
     <t xml:space="preserve">Štefan Nagy Bačo</t>
   </si>
   <si>
+    <t xml:space="preserve">Pôžička – BauHausEurope s.r.o. pre PSPSK s.r.o.</t>
+  </si>
+  <si>
     <t xml:space="preserve">áno</t>
   </si>
   <si>
     <t xml:space="preserve">otvorené</t>
   </si>
   <si>
+    <t xml:space="preserve">Pôžička v hotovosti v SL (december 2024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">presný deň neznámy – použitý 31.12.2024, DOPLŇTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nevrátená suma (11/2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">presný deň neznámy – použitý 30.11.2025, DOPLŇTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dvere – nedodané</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dvere – ďalšia platba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lukáš Cisco</t>
+  </si>
+  <si>
     <t xml:space="preserve">doplňte istinu a dátum</t>
   </si>
   <si>
-    <t xml:space="preserve">Lukáš Cisco</t>
-  </si>
-  <si>
     <t xml:space="preserve">Baláž</t>
   </si>
   <si>
@@ -177,19 +198,22 @@
     <t xml:space="preserve">bez úroku – doplňte istinu a dátum</t>
   </si>
   <si>
-    <t xml:space="preserve">PRÍKLAD – Ján Novák</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pôžička podľa zmluvy z 15.01.2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">príklad formátu – prepíšte / vymažte</t>
+    <t xml:space="preserve">YQ House</t>
+  </si>
+  <si>
+    <t xml:space="preserve">súvisí so Štefanom – doplňte istinu a dátum</t>
   </si>
   <si>
     <t xml:space="preserve">SPOLU – otvorené pohľadávky</t>
   </si>
   <si>
     <t xml:space="preserve">počet:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Súhrn podľa dlžníka (len otvorené pohľadávky)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pri novom dlžníkovi doplňte meno do stĺpca A v tomto súhrne – vzorce sú SUMIFS.</t>
   </si>
   <si>
     <t xml:space="preserve">Detailný rozpis úročenia pre jedného dlžníka (podklad do výzvy / žaloby)</t>
@@ -415,7 +439,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -489,6 +513,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -784,7 +816,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M62"/>
+  <dimension ref="A1:M69"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -906,120 +938,136 @@
       <c r="A11" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="10"/>
-      <c r="C11" s="11"/>
-      <c r="D11" s="12"/>
+      <c r="B11" s="10" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="11" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D11" s="12" t="n">
+        <v>45471</v>
+      </c>
       <c r="E11" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G11" s="13" t="str">
+        <v>27</v>
+      </c>
+      <c r="G11" s="13" t="n">
         <f aca="false">IF(OR($A11="",$D11="",$C11=""),"",MAX(0,$B$3-$D11))</f>
-        <v/>
-      </c>
-      <c r="H11" s="13" t="str">
+        <v>835</v>
+      </c>
+      <c r="H11" s="13" t="n">
         <f aca="false">IF($G11="","",IF(OR($E11="nie",$B$3&lt;=$D11),0,INT(DATEDIF($D11,$B$3,"m")/$B$5)))</f>
-        <v/>
-      </c>
-      <c r="I11" s="13" t="str">
+        <v>9</v>
+      </c>
+      <c r="I11" s="13" t="n">
         <f aca="false">IF($H11="","",IF($E11="nie",0,MAX(0,$B$3-EDATE($D11,$H11*$B$5))))</f>
-        <v/>
-      </c>
-      <c r="J11" s="14" t="str">
+        <v>13</v>
+      </c>
+      <c r="J11" s="14" t="n">
         <f aca="false">IF($H11="","",$C11*(1+$B$6)^$H11)</f>
-        <v/>
-      </c>
-      <c r="K11" s="14" t="str">
+        <v>62443.1484973833</v>
+      </c>
+      <c r="K11" s="14" t="n">
         <f aca="false">IF($H11="","",IF($E11="nie",0,$J11*(1+$B$4*$I11/365)-$C11))</f>
-        <v/>
-      </c>
-      <c r="L11" s="15" t="str">
+        <v>12665.5487523055</v>
+      </c>
+      <c r="L11" s="15" t="n">
         <f aca="false">IF($H11="","",$C11+$K11)</f>
-        <v/>
-      </c>
-      <c r="M11" s="10" t="s">
-        <v>27</v>
-      </c>
+        <v>62665.5487523055</v>
+      </c>
+      <c r="M11" s="10"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="10"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="12"/>
+      <c r="C12" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D12" s="12" t="n">
+        <v>45657</v>
+      </c>
       <c r="E12" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G12" s="13" t="str">
+        <v>27</v>
+      </c>
+      <c r="G12" s="13" t="n">
         <f aca="false">IF(OR($A12="",$D12="",$C12=""),"",MAX(0,$B$3-$D12))</f>
-        <v/>
-      </c>
-      <c r="H12" s="13" t="str">
+        <v>649</v>
+      </c>
+      <c r="H12" s="13" t="n">
         <f aca="false">IF($G12="","",IF(OR($E12="nie",$B$3&lt;=$D12),0,INT(DATEDIF($D12,$B$3,"m")/$B$5)))</f>
-        <v/>
-      </c>
-      <c r="I12" s="13" t="str">
+        <v>7</v>
+      </c>
+      <c r="I12" s="13" t="n">
         <f aca="false">IF($H12="","",IF($E12="nie",0,MAX(0,$B$3-EDATE($D12,$H12*$B$5))))</f>
-        <v/>
-      </c>
-      <c r="J12" s="14" t="str">
+        <v>11</v>
+      </c>
+      <c r="J12" s="14" t="n">
         <f aca="false">IF($H12="","",$C12*(1+$B$6)^$H12)</f>
-        <v/>
-      </c>
-      <c r="K12" s="14" t="str">
+        <v>5943.42876834106</v>
+      </c>
+      <c r="K12" s="14" t="n">
         <f aca="false">IF($H12="","",IF($E12="nie",0,$J12*(1+$B$4*$I12/365)-$C12))</f>
-        <v/>
-      </c>
-      <c r="L12" s="15" t="str">
+        <v>961.340471478527</v>
+      </c>
+      <c r="L12" s="15" t="n">
         <f aca="false">IF($H12="","",$C12+$K12)</f>
-        <v/>
+        <v>5961.34047147853</v>
       </c>
       <c r="M12" s="10" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="10"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="12"/>
+        <v>24</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D13" s="12" t="n">
+        <v>45991</v>
+      </c>
       <c r="E13" s="10" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G13" s="13" t="str">
+        <v>27</v>
+      </c>
+      <c r="G13" s="13" t="n">
         <f aca="false">IF(OR($A13="",$D13="",$C13=""),"",MAX(0,$B$3-$D13))</f>
-        <v/>
-      </c>
-      <c r="H13" s="13" t="str">
+        <v>315</v>
+      </c>
+      <c r="H13" s="13" t="n">
         <f aca="false">IF($G13="","",IF(OR($E13="nie",$B$3&lt;=$D13),0,INT(DATEDIF($D13,$B$3,"m")/$B$5)))</f>
-        <v/>
-      </c>
-      <c r="I13" s="13" t="str">
+        <v>3</v>
+      </c>
+      <c r="I13" s="13" t="n">
         <f aca="false">IF($H13="","",IF($E13="nie",0,MAX(0,$B$3-EDATE($D13,$H13*$B$5))))</f>
-        <v/>
-      </c>
-      <c r="J13" s="14" t="str">
+        <v>42</v>
+      </c>
+      <c r="J13" s="14" t="n">
         <f aca="false">IF($H13="","",$C13*(1+$B$6)^$H13)</f>
-        <v/>
-      </c>
-      <c r="K13" s="14" t="str">
+        <v>5384.453125</v>
+      </c>
+      <c r="K13" s="14" t="n">
         <f aca="false">IF($H13="","",IF($E13="nie",0,$J13*(1+$B$4*$I13/365)-$C13))</f>
-        <v/>
-      </c>
-      <c r="L13" s="15" t="str">
+        <v>446.411215753423</v>
+      </c>
+      <c r="L13" s="15" t="n">
         <f aca="false">IF($H13="","",$C13+$K13)</f>
-        <v/>
+        <v>5446.41121575342</v>
       </c>
       <c r="M13" s="10" t="s">
         <v>31</v>
@@ -1027,124 +1075,152 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B14" s="10" t="s">
-        <v>33</v>
-      </c>
       <c r="C14" s="11" t="n">
-        <v>5000</v>
+        <v>10000</v>
       </c>
       <c r="D14" s="12" t="n">
-        <v>45717</v>
+        <v>45830</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G14" s="13" t="n">
         <f aca="false">IF(OR($A14="",$D14="",$C14=""),"",MAX(0,$B$3-$D14))</f>
-        <v>589</v>
+        <v>476</v>
       </c>
       <c r="H14" s="13" t="n">
         <f aca="false">IF($G14="","",IF(OR($E14="nie",$B$3&lt;=$D14),0,INT(DATEDIF($D14,$B$3,"m")/$B$5)))</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I14" s="13" t="n">
         <f aca="false">IF($H14="","",IF($E14="nie",0,MAX(0,$B$3-EDATE($D14,$H14*$B$5))))</f>
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="J14" s="14" t="n">
         <f aca="false">IF($H14="","",$C14*(1+$B$6)^$H14)</f>
-        <v>5798.46709106445</v>
+        <v>11314.0821289062</v>
       </c>
       <c r="K14" s="14" t="n">
         <f aca="false">IF($H14="","",IF($E14="nie",0,$J14*(1+$B$4*$I14/365)-$C14))</f>
-        <v>862.011935898033</v>
+        <v>1372.97735094713</v>
       </c>
       <c r="L14" s="15" t="n">
         <f aca="false">IF($H14="","",$C14+$K14)</f>
-        <v>5862.01193589803</v>
-      </c>
-      <c r="M14" s="10" t="s">
+        <v>11372.9773509471</v>
+      </c>
+      <c r="M14" s="10"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D15" s="12" t="n">
+        <v>45854</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="G15" s="13" t="n">
+        <f aca="false">IF(OR($A15="",$D15="",$C15=""),"",MAX(0,$B$3-$D15))</f>
+        <v>452</v>
+      </c>
+      <c r="H15" s="13" t="n">
+        <f aca="false">IF($G15="","",IF(OR($E15="nie",$B$3&lt;=$D15),0,INT(DATEDIF($D15,$B$3,"m")/$B$5)))</f>
+        <v>4</v>
+      </c>
+      <c r="I15" s="13" t="n">
+        <f aca="false">IF($H15="","",IF($E15="nie",0,MAX(0,$B$3-EDATE($D15,$H15*$B$5))))</f>
+        <v>87</v>
+      </c>
+      <c r="J15" s="14" t="n">
+        <f aca="false">IF($H15="","",$C15*(1+$B$6)^$H15)</f>
+        <v>5519.064453125</v>
+      </c>
+      <c r="K15" s="14" t="n">
+        <f aca="false">IF($H15="","",IF($E15="nie",0,$J15*(1+$B$4*$I15/365)-$C15))</f>
+        <v>650.614756528251</v>
+      </c>
+      <c r="L15" s="15" t="n">
+        <f aca="false">IF($H15="","",$C15+$K15)</f>
+        <v>5650.61475652825</v>
+      </c>
+      <c r="M15" s="10"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C16" s="11" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D16" s="12" t="n">
+        <v>45916</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="G16" s="13" t="n">
+        <f aca="false">IF(OR($A16="",$D16="",$C16=""),"",MAX(0,$B$3-$D16))</f>
+        <v>390</v>
+      </c>
+      <c r="H16" s="13" t="n">
+        <f aca="false">IF($G16="","",IF(OR($E16="nie",$B$3&lt;=$D16),0,INT(DATEDIF($D16,$B$3,"m")/$B$5)))</f>
+        <v>4</v>
+      </c>
+      <c r="I16" s="13" t="n">
+        <f aca="false">IF($H16="","",IF($E16="nie",0,MAX(0,$B$3-EDATE($D16,$H16*$B$5))))</f>
+        <v>25</v>
+      </c>
+      <c r="J16" s="14" t="n">
+        <f aca="false">IF($H16="","",$C16*(1+$B$6)^$H16)</f>
+        <v>22076.2578125</v>
+      </c>
+      <c r="K16" s="14" t="n">
+        <f aca="false">IF($H16="","",IF($E16="nie",0,$J16*(1+$B$4*$I16/365)-$C16))</f>
+        <v>2227.46505779109</v>
+      </c>
+      <c r="L16" s="15" t="n">
+        <f aca="false">IF($H16="","",$C16+$K16)</f>
+        <v>22227.4650577911</v>
+      </c>
+      <c r="M16" s="10"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="13" t="str">
-        <f aca="false">IF(OR($A15="",$D15="",$C15=""),"",MAX(0,$B$3-$D15))</f>
-        <v/>
-      </c>
-      <c r="H15" s="13" t="str">
-        <f aca="false">IF($G15="","",IF(OR($E15="nie",$B$3&lt;=$D15),0,INT(DATEDIF($D15,$B$3,"m")/$B$5)))</f>
-        <v/>
-      </c>
-      <c r="I15" s="13" t="str">
-        <f aca="false">IF($H15="","",IF($E15="nie",0,MAX(0,$B$3-EDATE($D15,$H15*$B$5))))</f>
-        <v/>
-      </c>
-      <c r="J15" s="14" t="str">
-        <f aca="false">IF($H15="","",$C15*(1+$B$6)^$H15)</f>
-        <v/>
-      </c>
-      <c r="K15" s="14" t="str">
-        <f aca="false">IF($H15="","",IF($E15="nie",0,$J15*(1+$B$4*$I15/365)-$C15))</f>
-        <v/>
-      </c>
-      <c r="L15" s="15" t="str">
-        <f aca="false">IF($H15="","",$C15+$K15)</f>
-        <v/>
-      </c>
-      <c r="M15" s="10"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="13" t="str">
-        <f aca="false">IF(OR($A16="",$D16="",$C16=""),"",MAX(0,$B$3-$D16))</f>
-        <v/>
-      </c>
-      <c r="H16" s="13" t="str">
-        <f aca="false">IF($G16="","",IF(OR($E16="nie",$B$3&lt;=$D16),0,INT(DATEDIF($D16,$B$3,"m")/$B$5)))</f>
-        <v/>
-      </c>
-      <c r="I16" s="13" t="str">
-        <f aca="false">IF($H16="","",IF($E16="nie",0,MAX(0,$B$3-EDATE($D16,$H16*$B$5))))</f>
-        <v/>
-      </c>
-      <c r="J16" s="14" t="str">
-        <f aca="false">IF($H16="","",$C16*(1+$B$6)^$H16)</f>
-        <v/>
-      </c>
-      <c r="K16" s="14" t="str">
-        <f aca="false">IF($H16="","",IF($E16="nie",0,$J16*(1+$B$4*$I16/365)-$C16))</f>
-        <v/>
-      </c>
-      <c r="L16" s="15" t="str">
-        <f aca="false">IF($H16="","",$C16+$K16)</f>
-        <v/>
-      </c>
-      <c r="M16" s="10"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10"/>
       <c r="B17" s="10"/>
       <c r="C17" s="11"/>
       <c r="D17" s="12"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
+      <c r="E17" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="G17" s="13" t="str">
         <f aca="false">IF(OR($A17="",$D17="",$C17=""),"",MAX(0,$B$3-$D17))</f>
         <v/>
@@ -1169,15 +1245,23 @@
         <f aca="false">IF($H17="","",$C17+$K17)</f>
         <v/>
       </c>
-      <c r="M17" s="10"/>
+      <c r="M17" s="10" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10"/>
+      <c r="A18" s="10" t="s">
+        <v>36</v>
+      </c>
       <c r="B18" s="10"/>
       <c r="C18" s="11"/>
       <c r="D18" s="12"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
+      <c r="E18" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="F18" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="G18" s="13" t="str">
         <f aca="false">IF(OR($A18="",$D18="",$C18=""),"",MAX(0,$B$3-$D18))</f>
         <v/>
@@ -1202,15 +1286,23 @@
         <f aca="false">IF($H18="","",$C18+$K18)</f>
         <v/>
       </c>
-      <c r="M18" s="10"/>
+      <c r="M18" s="10" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10"/>
+      <c r="A19" s="10" t="s">
+        <v>39</v>
+      </c>
       <c r="B19" s="10"/>
       <c r="C19" s="11"/>
       <c r="D19" s="12"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
+      <c r="E19" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="G19" s="13" t="str">
         <f aca="false">IF(OR($A19="",$D19="",$C19=""),"",MAX(0,$B$3-$D19))</f>
         <v/>
@@ -1235,7 +1327,9 @@
         <f aca="false">IF($H19="","",$C19+$K19)</f>
         <v/>
       </c>
-      <c r="M19" s="10"/>
+      <c r="M19" s="10" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10"/>
@@ -2592,34 +2686,164 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="16" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B62" s="16"/>
       <c r="C62" s="17" t="n">
         <f aca="false">SUMIF($F$11:$F$60,"otvorené",C11:C60)</f>
-        <v>5000</v>
+        <v>95000</v>
       </c>
       <c r="D62" s="16"/>
       <c r="E62" s="16"/>
       <c r="F62" s="16" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="G62" s="18" t="n">
         <f aca="false">COUNTIFS($F$11:$F$60,"otvorené",$C$11:$C$60,"&lt;&gt;")</f>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H62" s="16"/>
       <c r="I62" s="16"/>
       <c r="J62" s="16"/>
       <c r="K62" s="17" t="n">
         <f aca="false">SUMIF($F$11:$F$60,"otvorené",K11:K60)</f>
-        <v>862.011935898033</v>
+        <v>18324.3576048039</v>
       </c>
       <c r="L62" s="17" t="n">
         <f aca="false">SUMIF($F$11:$F$60,"otvorené",L11:L60)</f>
-        <v>5862.01193589803</v>
+        <v>113324.357604804</v>
       </c>
       <c r="M62" s="16"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="M64" s="4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="B65" s="19"/>
+      <c r="C65" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="D65" s="19"/>
+      <c r="E65" s="19"/>
+      <c r="F65" s="19"/>
+      <c r="G65" s="19"/>
+      <c r="H65" s="19"/>
+      <c r="I65" s="19"/>
+      <c r="J65" s="19"/>
+      <c r="K65" s="19" t="s">
+        <v>21</v>
+      </c>
+      <c r="L65" s="19" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B66" s="20"/>
+      <c r="C66" s="14" t="n">
+        <f aca="false">SUMIFS(C$11:C$60,$A$11:$A$60,$A66,$F$11:$F$60,"otvorené")</f>
+        <v>95000</v>
+      </c>
+      <c r="D66" s="20"/>
+      <c r="E66" s="20"/>
+      <c r="F66" s="20"/>
+      <c r="G66" s="20"/>
+      <c r="H66" s="20"/>
+      <c r="I66" s="20"/>
+      <c r="J66" s="20"/>
+      <c r="K66" s="14" t="n">
+        <f aca="false">SUMIFS(K$11:K$60,$A$11:$A$60,$A66,$F$11:$F$60,"otvorené")</f>
+        <v>18324.3576048039</v>
+      </c>
+      <c r="L66" s="15" t="n">
+        <f aca="false">SUMIFS(L$11:L$60,$A$11:$A$60,$A66,$F$11:$F$60,"otvorené")</f>
+        <v>113324.357604804</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B67" s="20"/>
+      <c r="C67" s="14" t="n">
+        <f aca="false">SUMIFS(C$11:C$60,$A$11:$A$60,$A67,$F$11:$F$60,"otvorené")</f>
+        <v>0</v>
+      </c>
+      <c r="D67" s="20"/>
+      <c r="E67" s="20"/>
+      <c r="F67" s="20"/>
+      <c r="G67" s="20"/>
+      <c r="H67" s="20"/>
+      <c r="I67" s="20"/>
+      <c r="J67" s="20"/>
+      <c r="K67" s="14" t="n">
+        <f aca="false">SUMIFS(K$11:K$60,$A$11:$A$60,$A67,$F$11:$F$60,"otvorené")</f>
+        <v>0</v>
+      </c>
+      <c r="L67" s="15" t="n">
+        <f aca="false">SUMIFS(L$11:L$60,$A$11:$A$60,$A67,$F$11:$F$60,"otvorené")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="B68" s="20"/>
+      <c r="C68" s="14" t="n">
+        <f aca="false">SUMIFS(C$11:C$60,$A$11:$A$60,$A68,$F$11:$F$60,"otvorené")</f>
+        <v>0</v>
+      </c>
+      <c r="D68" s="20"/>
+      <c r="E68" s="20"/>
+      <c r="F68" s="20"/>
+      <c r="G68" s="20"/>
+      <c r="H68" s="20"/>
+      <c r="I68" s="20"/>
+      <c r="J68" s="20"/>
+      <c r="K68" s="14" t="n">
+        <f aca="false">SUMIFS(K$11:K$60,$A$11:$A$60,$A68,$F$11:$F$60,"otvorené")</f>
+        <v>0</v>
+      </c>
+      <c r="L68" s="15" t="n">
+        <f aca="false">SUMIFS(L$11:L$60,$A$11:$A$60,$A68,$F$11:$F$60,"otvorené")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="B69" s="20"/>
+      <c r="C69" s="14" t="n">
+        <f aca="false">SUMIFS(C$11:C$60,$A$11:$A$60,$A69,$F$11:$F$60,"otvorené")</f>
+        <v>0</v>
+      </c>
+      <c r="D69" s="20"/>
+      <c r="E69" s="20"/>
+      <c r="F69" s="20"/>
+      <c r="G69" s="20"/>
+      <c r="H69" s="20"/>
+      <c r="I69" s="20"/>
+      <c r="J69" s="20"/>
+      <c r="K69" s="14" t="n">
+        <f aca="false">SUMIFS(K$11:K$60,$A$11:$A$60,$A69,$F$11:$F$60,"otvorené")</f>
+        <v>0</v>
+      </c>
+      <c r="L69" s="15" t="n">
+        <f aca="false">SUMIFS(L$11:L$60,$A$11:$A$60,$A69,$F$11:$F$60,"otvorené")</f>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -2660,92 +2884,92 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="19" t="n">
+      <c r="B4" s="21" t="n">
         <f aca="false">INDEX('Súpis dlhov'!$C$11:$C$60,MATCH($B$3,'Súpis dlhov'!$A$11:$A$60,0))</f>
-        <v>5000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="B5" s="20" t="n">
+        <v>48</v>
+      </c>
+      <c r="B5" s="22" t="n">
         <f aca="false">INDEX('Súpis dlhov'!$D$11:$D$60,MATCH($B$3,'Súpis dlhov'!$A$11:$A$60,0))</f>
-        <v>45717</v>
+        <v>45471</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6" s="20" t="n">
+        <v>49</v>
+      </c>
+      <c r="B6" s="22" t="n">
         <f aca="false">'Súpis dlhov'!$B$3</f>
         <v>46306</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B7" s="21" t="n">
+        <v>50</v>
+      </c>
+      <c r="B7" s="23" t="n">
         <f aca="false">INDEX('Súpis dlhov'!$H$11:$H$60,MATCH($B$3,'Súpis dlhov'!$A$11:$A$60,0))</f>
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B8" s="22" t="n">
+        <v>51</v>
+      </c>
+      <c r="B8" s="24" t="n">
         <f aca="false">IF($B$9="nie",0,'Súpis dlhov'!$B$6)</f>
         <v>0.025</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="B9" s="23" t="str">
+        <v>52</v>
+      </c>
+      <c r="B9" s="25" t="str">
         <f aca="false">INDEX('Súpis dlhov'!$E$11:$E$60,MATCH($B$3,'Súpis dlhov'!$A$11:$A$60,0))</f>
         <v>áno</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2753,25 +2977,25 @@
         <f aca="false">IF(1&lt;=$B$7,1,"")</f>
         <v>1</v>
       </c>
-      <c r="B12" s="24" t="n">
+      <c r="B12" s="26" t="n">
         <f aca="false">IF($A12="","",EDATE($B$5,($A12-1)*'Súpis dlhov'!$B$5))</f>
-        <v>45717</v>
-      </c>
-      <c r="C12" s="24" t="n">
+        <v>45471</v>
+      </c>
+      <c r="C12" s="26" t="n">
         <f aca="false">IF($A12="","",EDATE($B$5,$A12*'Súpis dlhov'!$B$5))</f>
-        <v>45809</v>
+        <v>45563</v>
       </c>
       <c r="D12" s="14" t="n">
         <f aca="false">IF($A12="","",$B$4)</f>
-        <v>5000</v>
+        <v>50000</v>
       </c>
       <c r="E12" s="14" t="n">
         <f aca="false">IF($A12="","",$D12*$B$8)</f>
-        <v>125</v>
+        <v>1250</v>
       </c>
       <c r="F12" s="14" t="n">
         <f aca="false">IF($A12="","",$D12+$E12)</f>
-        <v>5125</v>
+        <v>51250</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2779,25 +3003,25 @@
         <f aca="false">IF(2&lt;=$B$7,2,"")</f>
         <v>2</v>
       </c>
-      <c r="B13" s="24" t="n">
+      <c r="B13" s="26" t="n">
         <f aca="false">IF($A13="","",EDATE($B$5,($A13-1)*'Súpis dlhov'!$B$5))</f>
-        <v>45809</v>
-      </c>
-      <c r="C13" s="24" t="n">
+        <v>45563</v>
+      </c>
+      <c r="C13" s="26" t="n">
         <f aca="false">IF($A13="","",EDATE($B$5,$A13*'Súpis dlhov'!$B$5))</f>
-        <v>45901</v>
+        <v>45654</v>
       </c>
       <c r="D13" s="14" t="n">
         <f aca="false">IF($A13="","",$F12)</f>
-        <v>5125</v>
+        <v>51250</v>
       </c>
       <c r="E13" s="14" t="n">
         <f aca="false">IF($A13="","",$D13*$B$8)</f>
-        <v>128.125</v>
+        <v>1281.25</v>
       </c>
       <c r="F13" s="14" t="n">
         <f aca="false">IF($A13="","",$D13+$E13)</f>
-        <v>5253.125</v>
+        <v>52531.25</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2805,25 +3029,25 @@
         <f aca="false">IF(3&lt;=$B$7,3,"")</f>
         <v>3</v>
       </c>
-      <c r="B14" s="24" t="n">
+      <c r="B14" s="26" t="n">
         <f aca="false">IF($A14="","",EDATE($B$5,($A14-1)*'Súpis dlhov'!$B$5))</f>
-        <v>45901</v>
-      </c>
-      <c r="C14" s="24" t="n">
+        <v>45654</v>
+      </c>
+      <c r="C14" s="26" t="n">
         <f aca="false">IF($A14="","",EDATE($B$5,$A14*'Súpis dlhov'!$B$5))</f>
-        <v>45992</v>
+        <v>45744</v>
       </c>
       <c r="D14" s="14" t="n">
         <f aca="false">IF($A14="","",$F13)</f>
-        <v>5253.125</v>
+        <v>52531.25</v>
       </c>
       <c r="E14" s="14" t="n">
         <f aca="false">IF($A14="","",$D14*$B$8)</f>
-        <v>131.328125</v>
+        <v>1313.28125</v>
       </c>
       <c r="F14" s="14" t="n">
         <f aca="false">IF($A14="","",$D14+$E14)</f>
-        <v>5384.453125</v>
+        <v>53844.53125</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2831,25 +3055,25 @@
         <f aca="false">IF(4&lt;=$B$7,4,"")</f>
         <v>4</v>
       </c>
-      <c r="B15" s="24" t="n">
+      <c r="B15" s="26" t="n">
         <f aca="false">IF($A15="","",EDATE($B$5,($A15-1)*'Súpis dlhov'!$B$5))</f>
-        <v>45992</v>
-      </c>
-      <c r="C15" s="24" t="n">
+        <v>45744</v>
+      </c>
+      <c r="C15" s="26" t="n">
         <f aca="false">IF($A15="","",EDATE($B$5,$A15*'Súpis dlhov'!$B$5))</f>
-        <v>46082</v>
+        <v>45836</v>
       </c>
       <c r="D15" s="14" t="n">
         <f aca="false">IF($A15="","",$F14)</f>
-        <v>5384.453125</v>
+        <v>53844.53125</v>
       </c>
       <c r="E15" s="14" t="n">
         <f aca="false">IF($A15="","",$D15*$B$8)</f>
-        <v>134.611328125</v>
+        <v>1346.11328125</v>
       </c>
       <c r="F15" s="14" t="n">
         <f aca="false">IF($A15="","",$D15+$E15)</f>
-        <v>5519.064453125</v>
+        <v>55190.64453125</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2857,25 +3081,25 @@
         <f aca="false">IF(5&lt;=$B$7,5,"")</f>
         <v>5</v>
       </c>
-      <c r="B16" s="24" t="n">
+      <c r="B16" s="26" t="n">
         <f aca="false">IF($A16="","",EDATE($B$5,($A16-1)*'Súpis dlhov'!$B$5))</f>
-        <v>46082</v>
-      </c>
-      <c r="C16" s="24" t="n">
+        <v>45836</v>
+      </c>
+      <c r="C16" s="26" t="n">
         <f aca="false">IF($A16="","",EDATE($B$5,$A16*'Súpis dlhov'!$B$5))</f>
-        <v>46174</v>
+        <v>45928</v>
       </c>
       <c r="D16" s="14" t="n">
         <f aca="false">IF($A16="","",$F15)</f>
-        <v>5519.064453125</v>
+        <v>55190.64453125</v>
       </c>
       <c r="E16" s="14" t="n">
         <f aca="false">IF($A16="","",$D16*$B$8)</f>
-        <v>137.976611328125</v>
+        <v>1379.76611328125</v>
       </c>
       <c r="F16" s="14" t="n">
         <f aca="false">IF($A16="","",$D16+$E16)</f>
-        <v>5657.04106445313</v>
+        <v>56570.4106445313</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2883,103 +3107,103 @@
         <f aca="false">IF(6&lt;=$B$7,6,"")</f>
         <v>6</v>
       </c>
-      <c r="B17" s="24" t="n">
+      <c r="B17" s="26" t="n">
         <f aca="false">IF($A17="","",EDATE($B$5,($A17-1)*'Súpis dlhov'!$B$5))</f>
-        <v>46174</v>
-      </c>
-      <c r="C17" s="24" t="n">
+        <v>45928</v>
+      </c>
+      <c r="C17" s="26" t="n">
         <f aca="false">IF($A17="","",EDATE($B$5,$A17*'Súpis dlhov'!$B$5))</f>
-        <v>46266</v>
+        <v>46019</v>
       </c>
       <c r="D17" s="14" t="n">
         <f aca="false">IF($A17="","",$F16)</f>
-        <v>5657.04106445313</v>
+        <v>56570.4106445313</v>
       </c>
       <c r="E17" s="14" t="n">
         <f aca="false">IF($A17="","",$D17*$B$8)</f>
-        <v>141.426026611328</v>
+        <v>1414.26026611328</v>
       </c>
       <c r="F17" s="14" t="n">
         <f aca="false">IF($A17="","",$D17+$E17)</f>
-        <v>5798.46709106445</v>
+        <v>57984.6709106445</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="str">
+      <c r="A18" s="13" t="n">
         <f aca="false">IF(7&lt;=$B$7,7,"")</f>
-        <v/>
-      </c>
-      <c r="B18" s="24" t="str">
+        <v>7</v>
+      </c>
+      <c r="B18" s="26" t="n">
         <f aca="false">IF($A18="","",EDATE($B$5,($A18-1)*'Súpis dlhov'!$B$5))</f>
-        <v/>
-      </c>
-      <c r="C18" s="24" t="str">
+        <v>46019</v>
+      </c>
+      <c r="C18" s="26" t="n">
         <f aca="false">IF($A18="","",EDATE($B$5,$A18*'Súpis dlhov'!$B$5))</f>
-        <v/>
-      </c>
-      <c r="D18" s="14" t="str">
+        <v>46109</v>
+      </c>
+      <c r="D18" s="14" t="n">
         <f aca="false">IF($A18="","",$F17)</f>
-        <v/>
-      </c>
-      <c r="E18" s="14" t="str">
+        <v>57984.6709106445</v>
+      </c>
+      <c r="E18" s="14" t="n">
         <f aca="false">IF($A18="","",$D18*$B$8)</f>
-        <v/>
-      </c>
-      <c r="F18" s="14" t="str">
+        <v>1449.61677276611</v>
+      </c>
+      <c r="F18" s="14" t="n">
         <f aca="false">IF($A18="","",$D18+$E18)</f>
-        <v/>
+        <v>59434.2876834107</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="str">
+      <c r="A19" s="13" t="n">
         <f aca="false">IF(8&lt;=$B$7,8,"")</f>
-        <v/>
-      </c>
-      <c r="B19" s="24" t="str">
+        <v>8</v>
+      </c>
+      <c r="B19" s="26" t="n">
         <f aca="false">IF($A19="","",EDATE($B$5,($A19-1)*'Súpis dlhov'!$B$5))</f>
-        <v/>
-      </c>
-      <c r="C19" s="24" t="str">
+        <v>46109</v>
+      </c>
+      <c r="C19" s="26" t="n">
         <f aca="false">IF($A19="","",EDATE($B$5,$A19*'Súpis dlhov'!$B$5))</f>
-        <v/>
-      </c>
-      <c r="D19" s="14" t="str">
+        <v>46201</v>
+      </c>
+      <c r="D19" s="14" t="n">
         <f aca="false">IF($A19="","",$F18)</f>
-        <v/>
-      </c>
-      <c r="E19" s="14" t="str">
+        <v>59434.2876834107</v>
+      </c>
+      <c r="E19" s="14" t="n">
         <f aca="false">IF($A19="","",$D19*$B$8)</f>
-        <v/>
-      </c>
-      <c r="F19" s="14" t="str">
+        <v>1485.85719208527</v>
+      </c>
+      <c r="F19" s="14" t="n">
         <f aca="false">IF($A19="","",$D19+$E19)</f>
-        <v/>
+        <v>60920.1448754959</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13" t="str">
+      <c r="A20" s="13" t="n">
         <f aca="false">IF(9&lt;=$B$7,9,"")</f>
-        <v/>
-      </c>
-      <c r="B20" s="24" t="str">
+        <v>9</v>
+      </c>
+      <c r="B20" s="26" t="n">
         <f aca="false">IF($A20="","",EDATE($B$5,($A20-1)*'Súpis dlhov'!$B$5))</f>
-        <v/>
-      </c>
-      <c r="C20" s="24" t="str">
+        <v>46201</v>
+      </c>
+      <c r="C20" s="26" t="n">
         <f aca="false">IF($A20="","",EDATE($B$5,$A20*'Súpis dlhov'!$B$5))</f>
-        <v/>
-      </c>
-      <c r="D20" s="14" t="str">
+        <v>46293</v>
+      </c>
+      <c r="D20" s="14" t="n">
         <f aca="false">IF($A20="","",$F19)</f>
-        <v/>
-      </c>
-      <c r="E20" s="14" t="str">
+        <v>60920.1448754959</v>
+      </c>
+      <c r="E20" s="14" t="n">
         <f aca="false">IF($A20="","",$D20*$B$8)</f>
-        <v/>
-      </c>
-      <c r="F20" s="14" t="str">
+        <v>1523.0036218874</v>
+      </c>
+      <c r="F20" s="14" t="n">
         <f aca="false">IF($A20="","",$D20+$E20)</f>
-        <v/>
+        <v>62443.1484973833</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2987,11 +3211,11 @@
         <f aca="false">IF(10&lt;=$B$7,10,"")</f>
         <v/>
       </c>
-      <c r="B21" s="24" t="str">
+      <c r="B21" s="26" t="str">
         <f aca="false">IF($A21="","",EDATE($B$5,($A21-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C21" s="24" t="str">
+      <c r="C21" s="26" t="str">
         <f aca="false">IF($A21="","",EDATE($B$5,$A21*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3013,11 +3237,11 @@
         <f aca="false">IF(11&lt;=$B$7,11,"")</f>
         <v/>
       </c>
-      <c r="B22" s="24" t="str">
+      <c r="B22" s="26" t="str">
         <f aca="false">IF($A22="","",EDATE($B$5,($A22-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C22" s="24" t="str">
+      <c r="C22" s="26" t="str">
         <f aca="false">IF($A22="","",EDATE($B$5,$A22*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3039,11 +3263,11 @@
         <f aca="false">IF(12&lt;=$B$7,12,"")</f>
         <v/>
       </c>
-      <c r="B23" s="24" t="str">
+      <c r="B23" s="26" t="str">
         <f aca="false">IF($A23="","",EDATE($B$5,($A23-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C23" s="24" t="str">
+      <c r="C23" s="26" t="str">
         <f aca="false">IF($A23="","",EDATE($B$5,$A23*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3065,11 +3289,11 @@
         <f aca="false">IF(13&lt;=$B$7,13,"")</f>
         <v/>
       </c>
-      <c r="B24" s="24" t="str">
+      <c r="B24" s="26" t="str">
         <f aca="false">IF($A24="","",EDATE($B$5,($A24-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C24" s="24" t="str">
+      <c r="C24" s="26" t="str">
         <f aca="false">IF($A24="","",EDATE($B$5,$A24*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3091,11 +3315,11 @@
         <f aca="false">IF(14&lt;=$B$7,14,"")</f>
         <v/>
       </c>
-      <c r="B25" s="24" t="str">
+      <c r="B25" s="26" t="str">
         <f aca="false">IF($A25="","",EDATE($B$5,($A25-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C25" s="24" t="str">
+      <c r="C25" s="26" t="str">
         <f aca="false">IF($A25="","",EDATE($B$5,$A25*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3117,11 +3341,11 @@
         <f aca="false">IF(15&lt;=$B$7,15,"")</f>
         <v/>
       </c>
-      <c r="B26" s="24" t="str">
+      <c r="B26" s="26" t="str">
         <f aca="false">IF($A26="","",EDATE($B$5,($A26-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C26" s="24" t="str">
+      <c r="C26" s="26" t="str">
         <f aca="false">IF($A26="","",EDATE($B$5,$A26*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3143,11 +3367,11 @@
         <f aca="false">IF(16&lt;=$B$7,16,"")</f>
         <v/>
       </c>
-      <c r="B27" s="24" t="str">
+      <c r="B27" s="26" t="str">
         <f aca="false">IF($A27="","",EDATE($B$5,($A27-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C27" s="24" t="str">
+      <c r="C27" s="26" t="str">
         <f aca="false">IF($A27="","",EDATE($B$5,$A27*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3169,11 +3393,11 @@
         <f aca="false">IF(17&lt;=$B$7,17,"")</f>
         <v/>
       </c>
-      <c r="B28" s="24" t="str">
+      <c r="B28" s="26" t="str">
         <f aca="false">IF($A28="","",EDATE($B$5,($A28-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C28" s="24" t="str">
+      <c r="C28" s="26" t="str">
         <f aca="false">IF($A28="","",EDATE($B$5,$A28*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3195,11 +3419,11 @@
         <f aca="false">IF(18&lt;=$B$7,18,"")</f>
         <v/>
       </c>
-      <c r="B29" s="24" t="str">
+      <c r="B29" s="26" t="str">
         <f aca="false">IF($A29="","",EDATE($B$5,($A29-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C29" s="24" t="str">
+      <c r="C29" s="26" t="str">
         <f aca="false">IF($A29="","",EDATE($B$5,$A29*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3221,11 +3445,11 @@
         <f aca="false">IF(19&lt;=$B$7,19,"")</f>
         <v/>
       </c>
-      <c r="B30" s="24" t="str">
+      <c r="B30" s="26" t="str">
         <f aca="false">IF($A30="","",EDATE($B$5,($A30-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C30" s="24" t="str">
+      <c r="C30" s="26" t="str">
         <f aca="false">IF($A30="","",EDATE($B$5,$A30*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3247,11 +3471,11 @@
         <f aca="false">IF(20&lt;=$B$7,20,"")</f>
         <v/>
       </c>
-      <c r="B31" s="24" t="str">
+      <c r="B31" s="26" t="str">
         <f aca="false">IF($A31="","",EDATE($B$5,($A31-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C31" s="24" t="str">
+      <c r="C31" s="26" t="str">
         <f aca="false">IF($A31="","",EDATE($B$5,$A31*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3273,11 +3497,11 @@
         <f aca="false">IF(21&lt;=$B$7,21,"")</f>
         <v/>
       </c>
-      <c r="B32" s="24" t="str">
+      <c r="B32" s="26" t="str">
         <f aca="false">IF($A32="","",EDATE($B$5,($A32-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C32" s="24" t="str">
+      <c r="C32" s="26" t="str">
         <f aca="false">IF($A32="","",EDATE($B$5,$A32*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3299,11 +3523,11 @@
         <f aca="false">IF(22&lt;=$B$7,22,"")</f>
         <v/>
       </c>
-      <c r="B33" s="24" t="str">
+      <c r="B33" s="26" t="str">
         <f aca="false">IF($A33="","",EDATE($B$5,($A33-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C33" s="24" t="str">
+      <c r="C33" s="26" t="str">
         <f aca="false">IF($A33="","",EDATE($B$5,$A33*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3325,11 +3549,11 @@
         <f aca="false">IF(23&lt;=$B$7,23,"")</f>
         <v/>
       </c>
-      <c r="B34" s="24" t="str">
+      <c r="B34" s="26" t="str">
         <f aca="false">IF($A34="","",EDATE($B$5,($A34-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C34" s="24" t="str">
+      <c r="C34" s="26" t="str">
         <f aca="false">IF($A34="","",EDATE($B$5,$A34*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3351,11 +3575,11 @@
         <f aca="false">IF(24&lt;=$B$7,24,"")</f>
         <v/>
       </c>
-      <c r="B35" s="24" t="str">
+      <c r="B35" s="26" t="str">
         <f aca="false">IF($A35="","",EDATE($B$5,($A35-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C35" s="24" t="str">
+      <c r="C35" s="26" t="str">
         <f aca="false">IF($A35="","",EDATE($B$5,$A35*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3377,11 +3601,11 @@
         <f aca="false">IF(25&lt;=$B$7,25,"")</f>
         <v/>
       </c>
-      <c r="B36" s="24" t="str">
+      <c r="B36" s="26" t="str">
         <f aca="false">IF($A36="","",EDATE($B$5,($A36-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C36" s="24" t="str">
+      <c r="C36" s="26" t="str">
         <f aca="false">IF($A36="","",EDATE($B$5,$A36*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3403,11 +3627,11 @@
         <f aca="false">IF(26&lt;=$B$7,26,"")</f>
         <v/>
       </c>
-      <c r="B37" s="24" t="str">
+      <c r="B37" s="26" t="str">
         <f aca="false">IF($A37="","",EDATE($B$5,($A37-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C37" s="24" t="str">
+      <c r="C37" s="26" t="str">
         <f aca="false">IF($A37="","",EDATE($B$5,$A37*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3429,11 +3653,11 @@
         <f aca="false">IF(27&lt;=$B$7,27,"")</f>
         <v/>
       </c>
-      <c r="B38" s="24" t="str">
+      <c r="B38" s="26" t="str">
         <f aca="false">IF($A38="","",EDATE($B$5,($A38-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C38" s="24" t="str">
+      <c r="C38" s="26" t="str">
         <f aca="false">IF($A38="","",EDATE($B$5,$A38*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3455,11 +3679,11 @@
         <f aca="false">IF(28&lt;=$B$7,28,"")</f>
         <v/>
       </c>
-      <c r="B39" s="24" t="str">
+      <c r="B39" s="26" t="str">
         <f aca="false">IF($A39="","",EDATE($B$5,($A39-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C39" s="24" t="str">
+      <c r="C39" s="26" t="str">
         <f aca="false">IF($A39="","",EDATE($B$5,$A39*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3481,11 +3705,11 @@
         <f aca="false">IF(29&lt;=$B$7,29,"")</f>
         <v/>
       </c>
-      <c r="B40" s="24" t="str">
+      <c r="B40" s="26" t="str">
         <f aca="false">IF($A40="","",EDATE($B$5,($A40-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C40" s="24" t="str">
+      <c r="C40" s="26" t="str">
         <f aca="false">IF($A40="","",EDATE($B$5,$A40*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3507,11 +3731,11 @@
         <f aca="false">IF(30&lt;=$B$7,30,"")</f>
         <v/>
       </c>
-      <c r="B41" s="24" t="str">
+      <c r="B41" s="26" t="str">
         <f aca="false">IF($A41="","",EDATE($B$5,($A41-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C41" s="24" t="str">
+      <c r="C41" s="26" t="str">
         <f aca="false">IF($A41="","",EDATE($B$5,$A41*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3533,11 +3757,11 @@
         <f aca="false">IF(31&lt;=$B$7,31,"")</f>
         <v/>
       </c>
-      <c r="B42" s="24" t="str">
+      <c r="B42" s="26" t="str">
         <f aca="false">IF($A42="","",EDATE($B$5,($A42-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C42" s="24" t="str">
+      <c r="C42" s="26" t="str">
         <f aca="false">IF($A42="","",EDATE($B$5,$A42*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3559,11 +3783,11 @@
         <f aca="false">IF(32&lt;=$B$7,32,"")</f>
         <v/>
       </c>
-      <c r="B43" s="24" t="str">
+      <c r="B43" s="26" t="str">
         <f aca="false">IF($A43="","",EDATE($B$5,($A43-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C43" s="24" t="str">
+      <c r="C43" s="26" t="str">
         <f aca="false">IF($A43="","",EDATE($B$5,$A43*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3585,11 +3809,11 @@
         <f aca="false">IF(33&lt;=$B$7,33,"")</f>
         <v/>
       </c>
-      <c r="B44" s="24" t="str">
+      <c r="B44" s="26" t="str">
         <f aca="false">IF($A44="","",EDATE($B$5,($A44-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C44" s="24" t="str">
+      <c r="C44" s="26" t="str">
         <f aca="false">IF($A44="","",EDATE($B$5,$A44*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3611,11 +3835,11 @@
         <f aca="false">IF(34&lt;=$B$7,34,"")</f>
         <v/>
       </c>
-      <c r="B45" s="24" t="str">
+      <c r="B45" s="26" t="str">
         <f aca="false">IF($A45="","",EDATE($B$5,($A45-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C45" s="24" t="str">
+      <c r="C45" s="26" t="str">
         <f aca="false">IF($A45="","",EDATE($B$5,$A45*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3637,11 +3861,11 @@
         <f aca="false">IF(35&lt;=$B$7,35,"")</f>
         <v/>
       </c>
-      <c r="B46" s="24" t="str">
+      <c r="B46" s="26" t="str">
         <f aca="false">IF($A46="","",EDATE($B$5,($A46-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C46" s="24" t="str">
+      <c r="C46" s="26" t="str">
         <f aca="false">IF($A46="","",EDATE($B$5,$A46*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3663,11 +3887,11 @@
         <f aca="false">IF(36&lt;=$B$7,36,"")</f>
         <v/>
       </c>
-      <c r="B47" s="24" t="str">
+      <c r="B47" s="26" t="str">
         <f aca="false">IF($A47="","",EDATE($B$5,($A47-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C47" s="24" t="str">
+      <c r="C47" s="26" t="str">
         <f aca="false">IF($A47="","",EDATE($B$5,$A47*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3689,11 +3913,11 @@
         <f aca="false">IF(37&lt;=$B$7,37,"")</f>
         <v/>
       </c>
-      <c r="B48" s="24" t="str">
+      <c r="B48" s="26" t="str">
         <f aca="false">IF($A48="","",EDATE($B$5,($A48-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C48" s="24" t="str">
+      <c r="C48" s="26" t="str">
         <f aca="false">IF($A48="","",EDATE($B$5,$A48*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3715,11 +3939,11 @@
         <f aca="false">IF(38&lt;=$B$7,38,"")</f>
         <v/>
       </c>
-      <c r="B49" s="24" t="str">
+      <c r="B49" s="26" t="str">
         <f aca="false">IF($A49="","",EDATE($B$5,($A49-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C49" s="24" t="str">
+      <c r="C49" s="26" t="str">
         <f aca="false">IF($A49="","",EDATE($B$5,$A49*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3741,11 +3965,11 @@
         <f aca="false">IF(39&lt;=$B$7,39,"")</f>
         <v/>
       </c>
-      <c r="B50" s="24" t="str">
+      <c r="B50" s="26" t="str">
         <f aca="false">IF($A50="","",EDATE($B$5,($A50-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C50" s="24" t="str">
+      <c r="C50" s="26" t="str">
         <f aca="false">IF($A50="","",EDATE($B$5,$A50*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3767,11 +3991,11 @@
         <f aca="false">IF(40&lt;=$B$7,40,"")</f>
         <v/>
       </c>
-      <c r="B51" s="24" t="str">
+      <c r="B51" s="26" t="str">
         <f aca="false">IF($A51="","",EDATE($B$5,($A51-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C51" s="24" t="str">
+      <c r="C51" s="26" t="str">
         <f aca="false">IF($A51="","",EDATE($B$5,$A51*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3793,11 +4017,11 @@
         <f aca="false">IF(41&lt;=$B$7,41,"")</f>
         <v/>
       </c>
-      <c r="B52" s="24" t="str">
+      <c r="B52" s="26" t="str">
         <f aca="false">IF($A52="","",EDATE($B$5,($A52-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C52" s="24" t="str">
+      <c r="C52" s="26" t="str">
         <f aca="false">IF($A52="","",EDATE($B$5,$A52*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3819,11 +4043,11 @@
         <f aca="false">IF(42&lt;=$B$7,42,"")</f>
         <v/>
       </c>
-      <c r="B53" s="24" t="str">
+      <c r="B53" s="26" t="str">
         <f aca="false">IF($A53="","",EDATE($B$5,($A53-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C53" s="24" t="str">
+      <c r="C53" s="26" t="str">
         <f aca="false">IF($A53="","",EDATE($B$5,$A53*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3845,11 +4069,11 @@
         <f aca="false">IF(43&lt;=$B$7,43,"")</f>
         <v/>
       </c>
-      <c r="B54" s="24" t="str">
+      <c r="B54" s="26" t="str">
         <f aca="false">IF($A54="","",EDATE($B$5,($A54-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C54" s="24" t="str">
+      <c r="C54" s="26" t="str">
         <f aca="false">IF($A54="","",EDATE($B$5,$A54*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3871,11 +4095,11 @@
         <f aca="false">IF(44&lt;=$B$7,44,"")</f>
         <v/>
       </c>
-      <c r="B55" s="24" t="str">
+      <c r="B55" s="26" t="str">
         <f aca="false">IF($A55="","",EDATE($B$5,($A55-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C55" s="24" t="str">
+      <c r="C55" s="26" t="str">
         <f aca="false">IF($A55="","",EDATE($B$5,$A55*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3897,11 +4121,11 @@
         <f aca="false">IF(45&lt;=$B$7,45,"")</f>
         <v/>
       </c>
-      <c r="B56" s="24" t="str">
+      <c r="B56" s="26" t="str">
         <f aca="false">IF($A56="","",EDATE($B$5,($A56-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C56" s="24" t="str">
+      <c r="C56" s="26" t="str">
         <f aca="false">IF($A56="","",EDATE($B$5,$A56*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3923,11 +4147,11 @@
         <f aca="false">IF(46&lt;=$B$7,46,"")</f>
         <v/>
       </c>
-      <c r="B57" s="24" t="str">
+      <c r="B57" s="26" t="str">
         <f aca="false">IF($A57="","",EDATE($B$5,($A57-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C57" s="24" t="str">
+      <c r="C57" s="26" t="str">
         <f aca="false">IF($A57="","",EDATE($B$5,$A57*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3949,11 +4173,11 @@
         <f aca="false">IF(47&lt;=$B$7,47,"")</f>
         <v/>
       </c>
-      <c r="B58" s="24" t="str">
+      <c r="B58" s="26" t="str">
         <f aca="false">IF($A58="","",EDATE($B$5,($A58-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C58" s="24" t="str">
+      <c r="C58" s="26" t="str">
         <f aca="false">IF($A58="","",EDATE($B$5,$A58*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -3975,11 +4199,11 @@
         <f aca="false">IF(48&lt;=$B$7,48,"")</f>
         <v/>
       </c>
-      <c r="B59" s="24" t="str">
+      <c r="B59" s="26" t="str">
         <f aca="false">IF($A59="","",EDATE($B$5,($A59-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C59" s="24" t="str">
+      <c r="C59" s="26" t="str">
         <f aca="false">IF($A59="","",EDATE($B$5,$A59*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4001,11 +4225,11 @@
         <f aca="false">IF(49&lt;=$B$7,49,"")</f>
         <v/>
       </c>
-      <c r="B60" s="24" t="str">
+      <c r="B60" s="26" t="str">
         <f aca="false">IF($A60="","",EDATE($B$5,($A60-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C60" s="24" t="str">
+      <c r="C60" s="26" t="str">
         <f aca="false">IF($A60="","",EDATE($B$5,$A60*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4027,11 +4251,11 @@
         <f aca="false">IF(50&lt;=$B$7,50,"")</f>
         <v/>
       </c>
-      <c r="B61" s="24" t="str">
+      <c r="B61" s="26" t="str">
         <f aca="false">IF($A61="","",EDATE($B$5,($A61-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C61" s="24" t="str">
+      <c r="C61" s="26" t="str">
         <f aca="false">IF($A61="","",EDATE($B$5,$A61*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4053,11 +4277,11 @@
         <f aca="false">IF(51&lt;=$B$7,51,"")</f>
         <v/>
       </c>
-      <c r="B62" s="24" t="str">
+      <c r="B62" s="26" t="str">
         <f aca="false">IF($A62="","",EDATE($B$5,($A62-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C62" s="24" t="str">
+      <c r="C62" s="26" t="str">
         <f aca="false">IF($A62="","",EDATE($B$5,$A62*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4079,11 +4303,11 @@
         <f aca="false">IF(52&lt;=$B$7,52,"")</f>
         <v/>
       </c>
-      <c r="B63" s="24" t="str">
+      <c r="B63" s="26" t="str">
         <f aca="false">IF($A63="","",EDATE($B$5,($A63-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C63" s="24" t="str">
+      <c r="C63" s="26" t="str">
         <f aca="false">IF($A63="","",EDATE($B$5,$A63*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4105,11 +4329,11 @@
         <f aca="false">IF(53&lt;=$B$7,53,"")</f>
         <v/>
       </c>
-      <c r="B64" s="24" t="str">
+      <c r="B64" s="26" t="str">
         <f aca="false">IF($A64="","",EDATE($B$5,($A64-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C64" s="24" t="str">
+      <c r="C64" s="26" t="str">
         <f aca="false">IF($A64="","",EDATE($B$5,$A64*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4131,11 +4355,11 @@
         <f aca="false">IF(54&lt;=$B$7,54,"")</f>
         <v/>
       </c>
-      <c r="B65" s="24" t="str">
+      <c r="B65" s="26" t="str">
         <f aca="false">IF($A65="","",EDATE($B$5,($A65-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C65" s="24" t="str">
+      <c r="C65" s="26" t="str">
         <f aca="false">IF($A65="","",EDATE($B$5,$A65*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4157,11 +4381,11 @@
         <f aca="false">IF(55&lt;=$B$7,55,"")</f>
         <v/>
       </c>
-      <c r="B66" s="24" t="str">
+      <c r="B66" s="26" t="str">
         <f aca="false">IF($A66="","",EDATE($B$5,($A66-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C66" s="24" t="str">
+      <c r="C66" s="26" t="str">
         <f aca="false">IF($A66="","",EDATE($B$5,$A66*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4183,11 +4407,11 @@
         <f aca="false">IF(56&lt;=$B$7,56,"")</f>
         <v/>
       </c>
-      <c r="B67" s="24" t="str">
+      <c r="B67" s="26" t="str">
         <f aca="false">IF($A67="","",EDATE($B$5,($A67-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C67" s="24" t="str">
+      <c r="C67" s="26" t="str">
         <f aca="false">IF($A67="","",EDATE($B$5,$A67*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4209,11 +4433,11 @@
         <f aca="false">IF(57&lt;=$B$7,57,"")</f>
         <v/>
       </c>
-      <c r="B68" s="24" t="str">
+      <c r="B68" s="26" t="str">
         <f aca="false">IF($A68="","",EDATE($B$5,($A68-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C68" s="24" t="str">
+      <c r="C68" s="26" t="str">
         <f aca="false">IF($A68="","",EDATE($B$5,$A68*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4235,11 +4459,11 @@
         <f aca="false">IF(58&lt;=$B$7,58,"")</f>
         <v/>
       </c>
-      <c r="B69" s="24" t="str">
+      <c r="B69" s="26" t="str">
         <f aca="false">IF($A69="","",EDATE($B$5,($A69-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C69" s="24" t="str">
+      <c r="C69" s="26" t="str">
         <f aca="false">IF($A69="","",EDATE($B$5,$A69*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4261,11 +4485,11 @@
         <f aca="false">IF(59&lt;=$B$7,59,"")</f>
         <v/>
       </c>
-      <c r="B70" s="24" t="str">
+      <c r="B70" s="26" t="str">
         <f aca="false">IF($A70="","",EDATE($B$5,($A70-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C70" s="24" t="str">
+      <c r="C70" s="26" t="str">
         <f aca="false">IF($A70="","",EDATE($B$5,$A70*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4287,11 +4511,11 @@
         <f aca="false">IF(60&lt;=$B$7,60,"")</f>
         <v/>
       </c>
-      <c r="B71" s="24" t="str">
+      <c r="B71" s="26" t="str">
         <f aca="false">IF($A71="","",EDATE($B$5,($A71-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C71" s="24" t="str">
+      <c r="C71" s="26" t="str">
         <f aca="false">IF($A71="","",EDATE($B$5,$A71*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4313,11 +4537,11 @@
         <f aca="false">IF(61&lt;=$B$7,61,"")</f>
         <v/>
       </c>
-      <c r="B72" s="24" t="str">
+      <c r="B72" s="26" t="str">
         <f aca="false">IF($A72="","",EDATE($B$5,($A72-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C72" s="24" t="str">
+      <c r="C72" s="26" t="str">
         <f aca="false">IF($A72="","",EDATE($B$5,$A72*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4339,11 +4563,11 @@
         <f aca="false">IF(62&lt;=$B$7,62,"")</f>
         <v/>
       </c>
-      <c r="B73" s="24" t="str">
+      <c r="B73" s="26" t="str">
         <f aca="false">IF($A73="","",EDATE($B$5,($A73-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C73" s="24" t="str">
+      <c r="C73" s="26" t="str">
         <f aca="false">IF($A73="","",EDATE($B$5,$A73*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4365,11 +4589,11 @@
         <f aca="false">IF(63&lt;=$B$7,63,"")</f>
         <v/>
       </c>
-      <c r="B74" s="24" t="str">
+      <c r="B74" s="26" t="str">
         <f aca="false">IF($A74="","",EDATE($B$5,($A74-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C74" s="24" t="str">
+      <c r="C74" s="26" t="str">
         <f aca="false">IF($A74="","",EDATE($B$5,$A74*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4391,11 +4615,11 @@
         <f aca="false">IF(64&lt;=$B$7,64,"")</f>
         <v/>
       </c>
-      <c r="B75" s="24" t="str">
+      <c r="B75" s="26" t="str">
         <f aca="false">IF($A75="","",EDATE($B$5,($A75-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C75" s="24" t="str">
+      <c r="C75" s="26" t="str">
         <f aca="false">IF($A75="","",EDATE($B$5,$A75*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4417,11 +4641,11 @@
         <f aca="false">IF(65&lt;=$B$7,65,"")</f>
         <v/>
       </c>
-      <c r="B76" s="24" t="str">
+      <c r="B76" s="26" t="str">
         <f aca="false">IF($A76="","",EDATE($B$5,($A76-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C76" s="24" t="str">
+      <c r="C76" s="26" t="str">
         <f aca="false">IF($A76="","",EDATE($B$5,$A76*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4443,11 +4667,11 @@
         <f aca="false">IF(66&lt;=$B$7,66,"")</f>
         <v/>
       </c>
-      <c r="B77" s="24" t="str">
+      <c r="B77" s="26" t="str">
         <f aca="false">IF($A77="","",EDATE($B$5,($A77-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C77" s="24" t="str">
+      <c r="C77" s="26" t="str">
         <f aca="false">IF($A77="","",EDATE($B$5,$A77*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4469,11 +4693,11 @@
         <f aca="false">IF(67&lt;=$B$7,67,"")</f>
         <v/>
       </c>
-      <c r="B78" s="24" t="str">
+      <c r="B78" s="26" t="str">
         <f aca="false">IF($A78="","",EDATE($B$5,($A78-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C78" s="24" t="str">
+      <c r="C78" s="26" t="str">
         <f aca="false">IF($A78="","",EDATE($B$5,$A78*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4495,11 +4719,11 @@
         <f aca="false">IF(68&lt;=$B$7,68,"")</f>
         <v/>
       </c>
-      <c r="B79" s="24" t="str">
+      <c r="B79" s="26" t="str">
         <f aca="false">IF($A79="","",EDATE($B$5,($A79-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C79" s="24" t="str">
+      <c r="C79" s="26" t="str">
         <f aca="false">IF($A79="","",EDATE($B$5,$A79*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4521,11 +4745,11 @@
         <f aca="false">IF(69&lt;=$B$7,69,"")</f>
         <v/>
       </c>
-      <c r="B80" s="24" t="str">
+      <c r="B80" s="26" t="str">
         <f aca="false">IF($A80="","",EDATE($B$5,($A80-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C80" s="24" t="str">
+      <c r="C80" s="26" t="str">
         <f aca="false">IF($A80="","",EDATE($B$5,$A80*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4547,11 +4771,11 @@
         <f aca="false">IF(70&lt;=$B$7,70,"")</f>
         <v/>
       </c>
-      <c r="B81" s="24" t="str">
+      <c r="B81" s="26" t="str">
         <f aca="false">IF($A81="","",EDATE($B$5,($A81-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C81" s="24" t="str">
+      <c r="C81" s="26" t="str">
         <f aca="false">IF($A81="","",EDATE($B$5,$A81*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4573,11 +4797,11 @@
         <f aca="false">IF(71&lt;=$B$7,71,"")</f>
         <v/>
       </c>
-      <c r="B82" s="24" t="str">
+      <c r="B82" s="26" t="str">
         <f aca="false">IF($A82="","",EDATE($B$5,($A82-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C82" s="24" t="str">
+      <c r="C82" s="26" t="str">
         <f aca="false">IF($A82="","",EDATE($B$5,$A82*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4599,11 +4823,11 @@
         <f aca="false">IF(72&lt;=$B$7,72,"")</f>
         <v/>
       </c>
-      <c r="B83" s="24" t="str">
+      <c r="B83" s="26" t="str">
         <f aca="false">IF($A83="","",EDATE($B$5,($A83-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C83" s="24" t="str">
+      <c r="C83" s="26" t="str">
         <f aca="false">IF($A83="","",EDATE($B$5,$A83*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4625,11 +4849,11 @@
         <f aca="false">IF(73&lt;=$B$7,73,"")</f>
         <v/>
       </c>
-      <c r="B84" s="24" t="str">
+      <c r="B84" s="26" t="str">
         <f aca="false">IF($A84="","",EDATE($B$5,($A84-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C84" s="24" t="str">
+      <c r="C84" s="26" t="str">
         <f aca="false">IF($A84="","",EDATE($B$5,$A84*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4651,11 +4875,11 @@
         <f aca="false">IF(74&lt;=$B$7,74,"")</f>
         <v/>
       </c>
-      <c r="B85" s="24" t="str">
+      <c r="B85" s="26" t="str">
         <f aca="false">IF($A85="","",EDATE($B$5,($A85-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C85" s="24" t="str">
+      <c r="C85" s="26" t="str">
         <f aca="false">IF($A85="","",EDATE($B$5,$A85*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4677,11 +4901,11 @@
         <f aca="false">IF(75&lt;=$B$7,75,"")</f>
         <v/>
       </c>
-      <c r="B86" s="24" t="str">
+      <c r="B86" s="26" t="str">
         <f aca="false">IF($A86="","",EDATE($B$5,($A86-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C86" s="24" t="str">
+      <c r="C86" s="26" t="str">
         <f aca="false">IF($A86="","",EDATE($B$5,$A86*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4703,11 +4927,11 @@
         <f aca="false">IF(76&lt;=$B$7,76,"")</f>
         <v/>
       </c>
-      <c r="B87" s="24" t="str">
+      <c r="B87" s="26" t="str">
         <f aca="false">IF($A87="","",EDATE($B$5,($A87-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C87" s="24" t="str">
+      <c r="C87" s="26" t="str">
         <f aca="false">IF($A87="","",EDATE($B$5,$A87*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4729,11 +4953,11 @@
         <f aca="false">IF(77&lt;=$B$7,77,"")</f>
         <v/>
       </c>
-      <c r="B88" s="24" t="str">
+      <c r="B88" s="26" t="str">
         <f aca="false">IF($A88="","",EDATE($B$5,($A88-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C88" s="24" t="str">
+      <c r="C88" s="26" t="str">
         <f aca="false">IF($A88="","",EDATE($B$5,$A88*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4755,11 +4979,11 @@
         <f aca="false">IF(78&lt;=$B$7,78,"")</f>
         <v/>
       </c>
-      <c r="B89" s="24" t="str">
+      <c r="B89" s="26" t="str">
         <f aca="false">IF($A89="","",EDATE($B$5,($A89-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C89" s="24" t="str">
+      <c r="C89" s="26" t="str">
         <f aca="false">IF($A89="","",EDATE($B$5,$A89*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4781,11 +5005,11 @@
         <f aca="false">IF(79&lt;=$B$7,79,"")</f>
         <v/>
       </c>
-      <c r="B90" s="24" t="str">
+      <c r="B90" s="26" t="str">
         <f aca="false">IF($A90="","",EDATE($B$5,($A90-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C90" s="24" t="str">
+      <c r="C90" s="26" t="str">
         <f aca="false">IF($A90="","",EDATE($B$5,$A90*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4807,11 +5031,11 @@
         <f aca="false">IF(80&lt;=$B$7,80,"")</f>
         <v/>
       </c>
-      <c r="B91" s="24" t="str">
+      <c r="B91" s="26" t="str">
         <f aca="false">IF($A91="","",EDATE($B$5,($A91-1)*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
-      <c r="C91" s="24" t="str">
+      <c r="C91" s="26" t="str">
         <f aca="false">IF($A91="","",EDATE($B$5,$A91*'Súpis dlhov'!$B$5))</f>
         <v/>
       </c>
@@ -4830,98 +5054,98 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="B93" s="25" t="n">
+        <v>59</v>
+      </c>
+      <c r="B93" s="27" t="n">
         <f aca="false">EDATE($B$5,$B$7*'Súpis dlhov'!$B$5)</f>
-        <v>46266</v>
-      </c>
-      <c r="C93" s="25" t="n">
+        <v>46293</v>
+      </c>
+      <c r="C93" s="27" t="n">
         <f aca="false">$B$6</f>
         <v>46306</v>
       </c>
-      <c r="D93" s="26" t="n">
+      <c r="D93" s="28" t="n">
         <f aca="false">IF($B$7=0,$B$4,INDEX($F$12:$F$91,$B$7))</f>
-        <v>5798.46709106445</v>
-      </c>
-      <c r="E93" s="26" t="n">
+        <v>62443.1484973833</v>
+      </c>
+      <c r="E93" s="28" t="n">
         <f aca="false">IF($B$9="nie",0,$D93*'Súpis dlhov'!$B$4*MAX(0,$C93-$B93)/365)</f>
-        <v>63.544844833583</v>
-      </c>
-      <c r="F93" s="26" t="n">
+        <v>222.400254922187</v>
+      </c>
+      <c r="F93" s="28" t="n">
         <f aca="false">$D93+$E93</f>
-        <v>5862.01193589804</v>
+        <v>62665.5487523055</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="B94" s="27" t="n">
+      <c r="B94" s="29" t="n">
         <f aca="false">MAX(0,$C93-$B93)</f>
-        <v>40</v>
-      </c>
-      <c r="C94" s="28"/>
-      <c r="D94" s="28"/>
-      <c r="E94" s="28"/>
-      <c r="F94" s="28"/>
+        <v>13</v>
+      </c>
+      <c r="C94" s="30"/>
+      <c r="D94" s="30"/>
+      <c r="E94" s="30"/>
+      <c r="F94" s="30"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="16"/>
-      <c r="B95" s="28"/>
-      <c r="C95" s="28"/>
-      <c r="D95" s="28"/>
-      <c r="E95" s="28"/>
-      <c r="F95" s="28"/>
+      <c r="B95" s="30"/>
+      <c r="C95" s="30"/>
+      <c r="D95" s="30"/>
+      <c r="E95" s="30"/>
+      <c r="F95" s="30"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="B96" s="28"/>
-      <c r="C96" s="28"/>
-      <c r="D96" s="28"/>
-      <c r="E96" s="28"/>
-      <c r="F96" s="26" t="n">
+      <c r="B96" s="30"/>
+      <c r="C96" s="30"/>
+      <c r="D96" s="30"/>
+      <c r="E96" s="30"/>
+      <c r="F96" s="28" t="n">
         <f aca="false">$B$4</f>
-        <v>5000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B97" s="28"/>
-      <c r="C97" s="28"/>
-      <c r="D97" s="28"/>
-      <c r="E97" s="28"/>
-      <c r="F97" s="26" t="n">
+      <c r="B97" s="30"/>
+      <c r="C97" s="30"/>
+      <c r="D97" s="30"/>
+      <c r="E97" s="30"/>
+      <c r="F97" s="28" t="n">
         <f aca="false">$F93-$B$4</f>
-        <v>862.011935898036</v>
+        <v>12665.5487523055</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="16" t="s">
-        <v>52</v>
-      </c>
-      <c r="B98" s="28"/>
-      <c r="C98" s="28"/>
-      <c r="D98" s="28"/>
-      <c r="E98" s="28"/>
+        <v>60</v>
+      </c>
+      <c r="B98" s="30"/>
+      <c r="C98" s="30"/>
+      <c r="D98" s="30"/>
+      <c r="E98" s="30"/>
       <c r="F98" s="17" t="n">
         <f aca="false">$F93</f>
-        <v>5862.01193589804</v>
+        <v>62665.5487523055</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="B99" s="28"/>
-      <c r="C99" s="28"/>
-      <c r="D99" s="28"/>
-      <c r="E99" s="28"/>
-      <c r="F99" s="26" t="n">
+        <v>61</v>
+      </c>
+      <c r="B99" s="30"/>
+      <c r="C99" s="30"/>
+      <c r="D99" s="30"/>
+      <c r="E99" s="30"/>
+      <c r="F99" s="28" t="n">
         <f aca="false">$F98-INDEX('Súpis dlhov'!$L$11:$L$60,MATCH($B$3,'Súpis dlhov'!$A$11:$A$60,0))</f>
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
Doplniť prenájom vozidla a doplatok za S-Class
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L5Qg2mKXdzeFPu6vSu8w6V
</commit_message>
<xml_diff>
--- a/supis_dlhov.xlsx
+++ b/supis_dlhov.xlsx
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="65">
   <si>
     <t xml:space="preserve">Súpis pohľadávok a výpočet úroku z omeškania</t>
   </si>
@@ -108,7 +108,7 @@
     <t xml:space="preserve">Vypočítané: 10 % × 3 / 12 = 2,5 % za štvrťrok.</t>
   </si>
   <si>
-    <t xml:space="preserve">Legenda: žlté bunky s modrým písmom vyplňte (dlžník, titul, istina, dátum, úročiť, stav, poznámka). Biele bunky sú vzorce – neprepisujte ich. Riadky 11–16 ukazujú formát vyplnenia (dátum DD.MM.RRRR, suma v €).</t>
+    <t xml:space="preserve">Legenda: žlté bunky s modrým písmom vyplňte (dlžník, titul, istina, dátum, úročiť, stav, poznámka). Biele bunky sú vzorce – neprepisujte ich. Riadky 11–18 ukazujú formát vyplnenia (dátum DD.MM.RRRR, suma v €).</t>
   </si>
   <si>
     <t xml:space="preserve">Metóda: za každé ukončené 3-mesačné obdobie od dátumu splatnosti sa úrok pripočíta k istine (zložené úročenie). Za nedokončené bežné obdobie sa počíta jednoduchý úrok z kapitalizovanej istiny pomerne podľa dní (rok = 365 dní). Pri „Úročiť = nie“ sa úrok nepočíta a dlžná suma = istina.</t>
@@ -181,6 +181,15 @@
   </si>
   <si>
     <t xml:space="preserve">Dvere – ďalšia platba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prenájom vozidla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dlžník neuvedený – priradené Bačovi, v prípade potreby zmeňte meno</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S-Class – uhradený doplatok</t>
   </si>
   <si>
     <t xml:space="preserve">Lukáš Cisco</t>
@@ -1210,40 +1219,46 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="B17" s="10"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="12"/>
+      <c r="C17" s="11" t="n">
+        <v>739.23</v>
+      </c>
+      <c r="D17" s="12" t="n">
+        <v>45798</v>
+      </c>
       <c r="E17" s="10" t="s">
         <v>26</v>
       </c>
       <c r="F17" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="G17" s="13" t="str">
+      <c r="G17" s="13" t="n">
         <f aca="false">IF(OR($A17="",$D17="",$C17=""),"",MAX(0,$B$3-$D17))</f>
-        <v/>
-      </c>
-      <c r="H17" s="13" t="str">
+        <v>508</v>
+      </c>
+      <c r="H17" s="13" t="n">
         <f aca="false">IF($G17="","",IF(OR($E17="nie",$B$3&lt;=$D17),0,INT(DATEDIF($D17,$B$3,"m")/$B$5)))</f>
-        <v/>
-      </c>
-      <c r="I17" s="13" t="str">
+        <v>5</v>
+      </c>
+      <c r="I17" s="13" t="n">
         <f aca="false">IF($H17="","",IF($E17="nie",0,MAX(0,$B$3-EDATE($D17,$H17*$B$5))))</f>
-        <v/>
-      </c>
-      <c r="J17" s="14" t="str">
+        <v>51</v>
+      </c>
+      <c r="J17" s="14" t="n">
         <f aca="false">IF($H17="","",$C17*(1+$B$6)^$H17)</f>
-        <v/>
-      </c>
-      <c r="K17" s="14" t="str">
+        <v>836.370893215136</v>
+      </c>
+      <c r="K17" s="14" t="n">
         <f aca="false">IF($H17="","",IF($E17="nie",0,$J17*(1+$B$4*$I17/365)-$C17))</f>
-        <v/>
-      </c>
-      <c r="L17" s="15" t="str">
+        <v>108.827171449101</v>
+      </c>
+      <c r="L17" s="15" t="n">
         <f aca="false">IF($H17="","",$C17+$K17)</f>
-        <v/>
+        <v>848.057171449101</v>
       </c>
       <c r="M17" s="10" t="s">
         <v>35</v>
@@ -1251,48 +1266,54 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B18" s="10"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="12"/>
+      <c r="C18" s="11" t="n">
+        <v>9692.15</v>
+      </c>
+      <c r="D18" s="12" t="n">
+        <v>45792</v>
+      </c>
       <c r="E18" s="10" t="s">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="F18" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="G18" s="13" t="str">
+      <c r="G18" s="13" t="n">
         <f aca="false">IF(OR($A18="",$D18="",$C18=""),"",MAX(0,$B$3-$D18))</f>
-        <v/>
-      </c>
-      <c r="H18" s="13" t="str">
+        <v>514</v>
+      </c>
+      <c r="H18" s="13" t="n">
         <f aca="false">IF($G18="","",IF(OR($E18="nie",$B$3&lt;=$D18),0,INT(DATEDIF($D18,$B$3,"m")/$B$5)))</f>
-        <v/>
-      </c>
-      <c r="I18" s="13" t="str">
+        <v>5</v>
+      </c>
+      <c r="I18" s="13" t="n">
         <f aca="false">IF($H18="","",IF($E18="nie",0,MAX(0,$B$3-EDATE($D18,$H18*$B$5))))</f>
-        <v/>
-      </c>
-      <c r="J18" s="14" t="str">
+        <v>57</v>
+      </c>
+      <c r="J18" s="14" t="n">
         <f aca="false">IF($H18="","",$C18*(1+$B$6)^$H18)</f>
-        <v/>
-      </c>
-      <c r="K18" s="14" t="str">
+        <v>10965.7781105679</v>
+      </c>
+      <c r="K18" s="14" t="n">
         <f aca="false">IF($H18="","",IF($E18="nie",0,$J18*(1+$B$4*$I18/365)-$C18))</f>
-        <v/>
-      </c>
-      <c r="L18" s="15" t="str">
+        <v>1444.87450845893</v>
+      </c>
+      <c r="L18" s="15" t="n">
         <f aca="false">IF($H18="","",$C18+$K18)</f>
-        <v/>
+        <v>11137.0245084589</v>
       </c>
       <c r="M18" s="10" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B19" s="10"/>
       <c r="C19" s="11"/>
@@ -1328,16 +1349,22 @@
         <v/>
       </c>
       <c r="M19" s="10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10"/>
+      <c r="A20" s="10" t="s">
+        <v>39</v>
+      </c>
       <c r="B20" s="10"/>
       <c r="C20" s="11"/>
       <c r="D20" s="12"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
+      <c r="E20" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="G20" s="13" t="str">
         <f aca="false">IF(OR($A20="",$D20="",$C20=""),"",MAX(0,$B$3-$D20))</f>
         <v/>
@@ -1362,15 +1389,23 @@
         <f aca="false">IF($H20="","",$C20+$K20)</f>
         <v/>
       </c>
-      <c r="M20" s="10"/>
+      <c r="M20" s="10" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10"/>
+      <c r="A21" s="10" t="s">
+        <v>42</v>
+      </c>
       <c r="B21" s="10"/>
       <c r="C21" s="11"/>
       <c r="D21" s="12"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
+      <c r="E21" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="G21" s="13" t="str">
         <f aca="false">IF(OR($A21="",$D21="",$C21=""),"",MAX(0,$B$3-$D21))</f>
         <v/>
@@ -1395,7 +1430,9 @@
         <f aca="false">IF($H21="","",$C21+$K21)</f>
         <v/>
       </c>
-      <c r="M21" s="10"/>
+      <c r="M21" s="10" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10"/>
@@ -2686,41 +2723,41 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="16" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B62" s="16"/>
       <c r="C62" s="17" t="n">
         <f aca="false">SUMIF($F$11:$F$60,"otvorené",C11:C60)</f>
-        <v>95000</v>
+        <v>105431.38</v>
       </c>
       <c r="D62" s="16"/>
       <c r="E62" s="16"/>
       <c r="F62" s="16" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="G62" s="18" t="n">
         <f aca="false">COUNTIFS($F$11:$F$60,"otvorené",$C$11:$C$60,"&lt;&gt;")</f>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H62" s="16"/>
       <c r="I62" s="16"/>
       <c r="J62" s="16"/>
       <c r="K62" s="17" t="n">
         <f aca="false">SUMIF($F$11:$F$60,"otvorené",K11:K60)</f>
-        <v>18324.3576048039</v>
+        <v>19878.0592847119</v>
       </c>
       <c r="L62" s="17" t="n">
         <f aca="false">SUMIF($F$11:$F$60,"otvorené",L11:L60)</f>
-        <v>113324.357604804</v>
+        <v>125309.439284712</v>
       </c>
       <c r="M62" s="16"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="M64" s="4" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2752,7 +2789,7 @@
       <c r="B66" s="20"/>
       <c r="C66" s="14" t="n">
         <f aca="false">SUMIFS(C$11:C$60,$A$11:$A$60,$A66,$F$11:$F$60,"otvorené")</f>
-        <v>95000</v>
+        <v>105431.38</v>
       </c>
       <c r="D66" s="20"/>
       <c r="E66" s="20"/>
@@ -2763,16 +2800,16 @@
       <c r="J66" s="20"/>
       <c r="K66" s="14" t="n">
         <f aca="false">SUMIFS(K$11:K$60,$A$11:$A$60,$A66,$F$11:$F$60,"otvorené")</f>
-        <v>18324.3576048039</v>
+        <v>19878.0592847119</v>
       </c>
       <c r="L66" s="15" t="n">
         <f aca="false">SUMIFS(L$11:L$60,$A$11:$A$60,$A66,$F$11:$F$60,"otvorené")</f>
-        <v>113324.357604804</v>
+        <v>125309.439284712</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="10" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B67" s="20"/>
       <c r="C67" s="14" t="n">
@@ -2797,7 +2834,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="10" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B68" s="20"/>
       <c r="C68" s="14" t="n">
@@ -2822,7 +2859,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="10" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B69" s="20"/>
       <c r="C69" s="14" t="n">
@@ -2884,18 +2921,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>24</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2909,7 +2946,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B5" s="22" t="n">
         <f aca="false">INDEX('Súpis dlhov'!$D$11:$D$60,MATCH($B$3,'Súpis dlhov'!$A$11:$A$60,0))</f>
@@ -2918,7 +2955,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B6" s="22" t="n">
         <f aca="false">'Súpis dlhov'!$B$3</f>
@@ -2927,7 +2964,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B7" s="23" t="n">
         <f aca="false">INDEX('Súpis dlhov'!$H$11:$H$60,MATCH($B$3,'Súpis dlhov'!$A$11:$A$60,0))</f>
@@ -2936,7 +2973,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B8" s="24" t="n">
         <f aca="false">IF($B$9="nie",0,'Súpis dlhov'!$B$6)</f>
@@ -2945,7 +2982,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B9" s="25" t="str">
         <f aca="false">INDEX('Súpis dlhov'!$E$11:$E$60,MATCH($B$3,'Súpis dlhov'!$A$11:$A$60,0))</f>
@@ -2954,22 +2991,22 @@
     </row>
     <row r="11" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5054,7 +5091,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="16" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B93" s="27" t="n">
         <f aca="false">EDATE($B$5,$B$7*'Súpis dlhov'!$B$5)</f>
@@ -5126,7 +5163,7 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="16" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B98" s="30"/>
       <c r="C98" s="30"/>
@@ -5139,7 +5176,7 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="16" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="B99" s="30"/>
       <c r="C99" s="30"/>

</xml_diff>

<commit_message>
Doplniť pohľadávky voči Lukášovi Ciscovi
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L5Qg2mKXdzeFPu6vSu8w6V
</commit_message>
<xml_diff>
--- a/supis_dlhov.xlsx
+++ b/supis_dlhov.xlsx
@@ -79,7 +79,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="71">
   <si>
     <t xml:space="preserve">Súpis pohľadávok a výpočet úroku z omeškania</t>
   </si>
@@ -108,7 +108,7 @@
     <t xml:space="preserve">Vypočítané: 10 % × 3 / 12 = 2,5 % za štvrťrok.</t>
   </si>
   <si>
-    <t xml:space="preserve">Legenda: žlté bunky s modrým písmom vyplňte (dlžník, titul, istina, dátum, úročiť, stav, poznámka). Biele bunky sú vzorce – neprepisujte ich. Riadky 11–18 ukazujú formát vyplnenia (dátum DD.MM.RRRR, suma v €).</t>
+    <t xml:space="preserve">Legenda: žlté bunky s modrým písmom vyplňte (dlžník, titul, istina, dátum, úročiť, stav, poznámka). Biele bunky sú vzorce – neprepisujte ich. Riadky 11–22 ukazujú formát vyplnenia (dátum DD.MM.RRRR, suma v €).</t>
   </si>
   <si>
     <t xml:space="preserve">Metóda: za každé ukončené 3-mesačné obdobie od dátumu splatnosti sa úrok pripočíta k istine (zložené úročenie). Za nedokončené bežné obdobie sa počíta jednoduchý úrok z kapitalizovanej istiny pomerne podľa dní (rok = 365 dní). Pri „Úročiť = nie“ sa úrok nepočíta a dlžná suma = istina.</t>
@@ -195,7 +195,25 @@
     <t xml:space="preserve">Lukáš Cisco</t>
   </si>
   <si>
-    <t xml:space="preserve">doplňte istinu a dátum</t>
+    <t xml:space="preserve">Prvá vlna (2022), cca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">suma približná, presný deň neznámy – použitý 31.12.2022, DOPLŇTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Druhá vlna (2024)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tretia vlna (2025)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">presný deň neznámy – použitý 31.12.2025, DOPLŇTE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Daň za rok 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dátum splatnosti neznámy – použitý 31.12.2025, DOPLŇTE</t>
   </si>
   <si>
     <t xml:space="preserve">Baláž</t>
@@ -1315,165 +1333,203 @@
       <c r="A19" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B19" s="10"/>
-      <c r="C19" s="11"/>
-      <c r="D19" s="12"/>
+      <c r="B19" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="C19" s="11" t="n">
+        <v>40000</v>
+      </c>
+      <c r="D19" s="12" t="n">
+        <v>44926</v>
+      </c>
       <c r="E19" s="10" t="s">
         <v>26</v>
       </c>
       <c r="F19" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="G19" s="13" t="str">
+      <c r="G19" s="13" t="n">
         <f aca="false">IF(OR($A19="",$D19="",$C19=""),"",MAX(0,$B$3-$D19))</f>
-        <v/>
-      </c>
-      <c r="H19" s="13" t="str">
+        <v>1380</v>
+      </c>
+      <c r="H19" s="13" t="n">
         <f aca="false">IF($G19="","",IF(OR($E19="nie",$B$3&lt;=$D19),0,INT(DATEDIF($D19,$B$3,"m")/$B$5)))</f>
-        <v/>
-      </c>
-      <c r="I19" s="13" t="str">
+        <v>15</v>
+      </c>
+      <c r="I19" s="13" t="n">
         <f aca="false">IF($H19="","",IF($E19="nie",0,MAX(0,$B$3-EDATE($D19,$H19*$B$5))))</f>
-        <v/>
-      </c>
-      <c r="J19" s="14" t="str">
+        <v>11</v>
+      </c>
+      <c r="J19" s="14" t="n">
         <f aca="false">IF($H19="","",$C19*(1+$B$6)^$H19)</f>
-        <v/>
-      </c>
-      <c r="K19" s="14" t="str">
+        <v>57931.9266599244</v>
+      </c>
+      <c r="K19" s="14" t="n">
         <f aca="false">IF($H19="","",IF($E19="nie",0,$J19*(1+$B$4*$I19/365)-$C19))</f>
-        <v/>
-      </c>
-      <c r="L19" s="15" t="str">
+        <v>18106.5160279406</v>
+      </c>
+      <c r="L19" s="15" t="n">
         <f aca="false">IF($H19="","",$C19+$K19)</f>
-        <v/>
+        <v>58106.5160279406</v>
       </c>
       <c r="M19" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="B20" s="10"/>
-      <c r="C20" s="11"/>
-      <c r="D20" s="12"/>
+        <v>37</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="11" t="n">
+        <v>30000</v>
+      </c>
+      <c r="D20" s="12" t="n">
+        <v>45657</v>
+      </c>
       <c r="E20" s="10" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="F20" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="G20" s="13" t="str">
+      <c r="G20" s="13" t="n">
         <f aca="false">IF(OR($A20="",$D20="",$C20=""),"",MAX(0,$B$3-$D20))</f>
-        <v/>
-      </c>
-      <c r="H20" s="13" t="str">
+        <v>649</v>
+      </c>
+      <c r="H20" s="13" t="n">
         <f aca="false">IF($G20="","",IF(OR($E20="nie",$B$3&lt;=$D20),0,INT(DATEDIF($D20,$B$3,"m")/$B$5)))</f>
-        <v/>
-      </c>
-      <c r="I20" s="13" t="str">
+        <v>7</v>
+      </c>
+      <c r="I20" s="13" t="n">
         <f aca="false">IF($H20="","",IF($E20="nie",0,MAX(0,$B$3-EDATE($D20,$H20*$B$5))))</f>
-        <v/>
-      </c>
-      <c r="J20" s="14" t="str">
+        <v>11</v>
+      </c>
+      <c r="J20" s="14" t="n">
         <f aca="false">IF($H20="","",$C20*(1+$B$6)^$H20)</f>
-        <v/>
-      </c>
-      <c r="K20" s="14" t="str">
+        <v>35660.5726100464</v>
+      </c>
+      <c r="K20" s="14" t="n">
         <f aca="false">IF($H20="","",IF($E20="nie",0,$J20*(1+$B$4*$I20/365)-$C20))</f>
-        <v/>
-      </c>
-      <c r="L20" s="15" t="str">
+        <v>5768.04282887116</v>
+      </c>
+      <c r="L20" s="15" t="n">
         <f aca="false">IF($H20="","",$C20+$K20)</f>
-        <v/>
+        <v>35768.0428288712</v>
       </c>
       <c r="M20" s="10" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="B21" s="10"/>
-      <c r="C21" s="11"/>
-      <c r="D21" s="12"/>
+        <v>37</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21" s="11" t="n">
+        <v>21000</v>
+      </c>
+      <c r="D21" s="12" t="n">
+        <v>46022</v>
+      </c>
       <c r="E21" s="10" t="s">
         <v>26</v>
       </c>
       <c r="F21" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="G21" s="13" t="str">
+      <c r="G21" s="13" t="n">
         <f aca="false">IF(OR($A21="",$D21="",$C21=""),"",MAX(0,$B$3-$D21))</f>
-        <v/>
-      </c>
-      <c r="H21" s="13" t="str">
+        <v>284</v>
+      </c>
+      <c r="H21" s="13" t="n">
         <f aca="false">IF($G21="","",IF(OR($E21="nie",$B$3&lt;=$D21),0,INT(DATEDIF($D21,$B$3,"m")/$B$5)))</f>
-        <v/>
-      </c>
-      <c r="I21" s="13" t="str">
+        <v>3</v>
+      </c>
+      <c r="I21" s="13" t="n">
         <f aca="false">IF($H21="","",IF($E21="nie",0,MAX(0,$B$3-EDATE($D21,$H21*$B$5))))</f>
-        <v/>
-      </c>
-      <c r="J21" s="14" t="str">
+        <v>11</v>
+      </c>
+      <c r="J21" s="14" t="n">
         <f aca="false">IF($H21="","",$C21*(1+$B$6)^$H21)</f>
-        <v/>
-      </c>
-      <c r="K21" s="14" t="str">
+        <v>22614.703125</v>
+      </c>
+      <c r="K21" s="14" t="n">
         <f aca="false">IF($H21="","",IF($E21="nie",0,$J21*(1+$B$4*$I21/365)-$C21))</f>
-        <v/>
-      </c>
-      <c r="L21" s="15" t="str">
+        <v>1682.85702482876</v>
+      </c>
+      <c r="L21" s="15" t="n">
         <f aca="false">IF($H21="","",$C21+$K21)</f>
-        <v/>
+        <v>22682.8570248288</v>
       </c>
       <c r="M21" s="10" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B22" s="10" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="11"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="13" t="str">
+      <c r="C22" s="11" t="n">
+        <v>35000</v>
+      </c>
+      <c r="D22" s="12" t="n">
+        <v>46022</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="G22" s="13" t="n">
         <f aca="false">IF(OR($A22="",$D22="",$C22=""),"",MAX(0,$B$3-$D22))</f>
-        <v/>
-      </c>
-      <c r="H22" s="13" t="str">
+        <v>284</v>
+      </c>
+      <c r="H22" s="13" t="n">
         <f aca="false">IF($G22="","",IF(OR($E22="nie",$B$3&lt;=$D22),0,INT(DATEDIF($D22,$B$3,"m")/$B$5)))</f>
-        <v/>
-      </c>
-      <c r="I22" s="13" t="str">
+        <v>3</v>
+      </c>
+      <c r="I22" s="13" t="n">
         <f aca="false">IF($H22="","",IF($E22="nie",0,MAX(0,$B$3-EDATE($D22,$H22*$B$5))))</f>
-        <v/>
-      </c>
-      <c r="J22" s="14" t="str">
+        <v>11</v>
+      </c>
+      <c r="J22" s="14" t="n">
         <f aca="false">IF($H22="","",$C22*(1+$B$6)^$H22)</f>
-        <v/>
-      </c>
-      <c r="K22" s="14" t="str">
+        <v>37691.171875</v>
+      </c>
+      <c r="K22" s="14" t="n">
         <f aca="false">IF($H22="","",IF($E22="nie",0,$J22*(1+$B$4*$I22/365)-$C22))</f>
-        <v/>
-      </c>
-      <c r="L22" s="15" t="str">
+        <v>2804.76170804793</v>
+      </c>
+      <c r="L22" s="15" t="n">
         <f aca="false">IF($H22="","",$C22+$K22)</f>
-        <v/>
-      </c>
-      <c r="M22" s="10"/>
+        <v>37804.7617080479</v>
+      </c>
+      <c r="M22" s="10" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10"/>
+      <c r="A23" s="10" t="s">
+        <v>45</v>
+      </c>
       <c r="B23" s="10"/>
       <c r="C23" s="11"/>
       <c r="D23" s="12"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
+      <c r="E23" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="G23" s="13" t="str">
         <f aca="false">IF(OR($A23="",$D23="",$C23=""),"",MAX(0,$B$3-$D23))</f>
         <v/>
@@ -1498,15 +1554,23 @@
         <f aca="false">IF($H23="","",$C23+$K23)</f>
         <v/>
       </c>
-      <c r="M23" s="10"/>
+      <c r="M23" s="10" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10"/>
+      <c r="A24" s="10" t="s">
+        <v>48</v>
+      </c>
       <c r="B24" s="10"/>
       <c r="C24" s="11"/>
       <c r="D24" s="12"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10"/>
+      <c r="E24" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>27</v>
+      </c>
       <c r="G24" s="13" t="str">
         <f aca="false">IF(OR($A24="",$D24="",$C24=""),"",MAX(0,$B$3-$D24))</f>
         <v/>
@@ -1531,7 +1595,9 @@
         <f aca="false">IF($H24="","",$C24+$K24)</f>
         <v/>
       </c>
-      <c r="M24" s="10"/>
+      <c r="M24" s="10" t="s">
+        <v>49</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10"/>
@@ -2723,41 +2789,41 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="16" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="B62" s="16"/>
       <c r="C62" s="17" t="n">
         <f aca="false">SUMIF($F$11:$F$60,"otvorené",C11:C60)</f>
-        <v>105431.38</v>
+        <v>231431.38</v>
       </c>
       <c r="D62" s="16"/>
       <c r="E62" s="16"/>
       <c r="F62" s="16" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="G62" s="18" t="n">
         <f aca="false">COUNTIFS($F$11:$F$60,"otvorené",$C$11:$C$60,"&lt;&gt;")</f>
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H62" s="16"/>
       <c r="I62" s="16"/>
       <c r="J62" s="16"/>
       <c r="K62" s="17" t="n">
         <f aca="false">SUMIF($F$11:$F$60,"otvorené",K11:K60)</f>
-        <v>19878.0592847119</v>
+        <v>48240.2368744004</v>
       </c>
       <c r="L62" s="17" t="n">
         <f aca="false">SUMIF($F$11:$F$60,"otvorené",L11:L60)</f>
-        <v>125309.439284712</v>
+        <v>279671.6168744</v>
       </c>
       <c r="M62" s="16"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="2" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="M64" s="4" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2814,7 +2880,7 @@
       <c r="B67" s="20"/>
       <c r="C67" s="14" t="n">
         <f aca="false">SUMIFS(C$11:C$60,$A$11:$A$60,$A67,$F$11:$F$60,"otvorené")</f>
-        <v>0</v>
+        <v>126000</v>
       </c>
       <c r="D67" s="20"/>
       <c r="E67" s="20"/>
@@ -2825,16 +2891,16 @@
       <c r="J67" s="20"/>
       <c r="K67" s="14" t="n">
         <f aca="false">SUMIFS(K$11:K$60,$A$11:$A$60,$A67,$F$11:$F$60,"otvorené")</f>
-        <v>0</v>
+        <v>28362.1775896885</v>
       </c>
       <c r="L67" s="15" t="n">
         <f aca="false">SUMIFS(L$11:L$60,$A$11:$A$60,$A67,$F$11:$F$60,"otvorené")</f>
-        <v>0</v>
+        <v>154362.177589688</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="10" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="B68" s="20"/>
       <c r="C68" s="14" t="n">
@@ -2859,7 +2925,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="10" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="B69" s="20"/>
       <c r="C69" s="14" t="n">
@@ -2921,18 +2987,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="B3" s="10" t="s">
         <v>24</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2946,7 +3012,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="B5" s="22" t="n">
         <f aca="false">INDEX('Súpis dlhov'!$D$11:$D$60,MATCH($B$3,'Súpis dlhov'!$A$11:$A$60,0))</f>
@@ -2955,7 +3021,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="B6" s="22" t="n">
         <f aca="false">'Súpis dlhov'!$B$3</f>
@@ -2964,7 +3030,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="B7" s="23" t="n">
         <f aca="false">INDEX('Súpis dlhov'!$H$11:$H$60,MATCH($B$3,'Súpis dlhov'!$A$11:$A$60,0))</f>
@@ -2973,7 +3039,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="B8" s="24" t="n">
         <f aca="false">IF($B$9="nie",0,'Súpis dlhov'!$B$6)</f>
@@ -2982,7 +3048,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="B9" s="25" t="str">
         <f aca="false">INDEX('Súpis dlhov'!$E$11:$E$60,MATCH($B$3,'Súpis dlhov'!$A$11:$A$60,0))</f>
@@ -2991,22 +3057,22 @@
     </row>
     <row r="11" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="F11" s="9" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5091,7 +5157,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="16" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B93" s="27" t="n">
         <f aca="false">EDATE($B$5,$B$7*'Súpis dlhov'!$B$5)</f>
@@ -5163,7 +5229,7 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="16" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="B98" s="30"/>
       <c r="C98" s="30"/>
@@ -5176,7 +5242,7 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="16" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="B99" s="30"/>
       <c r="C99" s="30"/>

</xml_diff>

<commit_message>
Upraviť daň za rok 2025 u Lukáša Cisca na 61 907 €
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L5Qg2mKXdzeFPu6vSu8w6V
</commit_message>
<xml_diff>
--- a/supis_dlhov.xlsx
+++ b/supis_dlhov.xlsx
@@ -1478,7 +1478,7 @@
         <v>43</v>
       </c>
       <c r="C22" s="11" t="n">
-        <v>35000</v>
+        <v>61907</v>
       </c>
       <c r="D22" s="12" t="n">
         <v>46022</v>
@@ -1503,15 +1503,15 @@
       </c>
       <c r="J22" s="14" t="n">
         <f aca="false">IF($H22="","",$C22*(1+$B$6)^$H22)</f>
-        <v>37691.171875</v>
+        <v>66667.067921875</v>
       </c>
       <c r="K22" s="14" t="n">
         <f aca="false">IF($H22="","",IF($E22="nie",0,$J22*(1+$B$4*$I22/365)-$C22))</f>
-        <v>2804.76170804793</v>
+        <v>4960.98237314638</v>
       </c>
       <c r="L22" s="15" t="n">
         <f aca="false">IF($H22="","",$C22+$K22)</f>
-        <v>37804.7617080479</v>
+        <v>66867.9823731464</v>
       </c>
       <c r="M22" s="10" t="s">
         <v>44</v>
@@ -2794,7 +2794,7 @@
       <c r="B62" s="16"/>
       <c r="C62" s="17" t="n">
         <f aca="false">SUMIF($F$11:$F$60,"otvorené",C11:C60)</f>
-        <v>231431.38</v>
+        <v>258338.38</v>
       </c>
       <c r="D62" s="16"/>
       <c r="E62" s="16"/>
@@ -2810,11 +2810,11 @@
       <c r="J62" s="16"/>
       <c r="K62" s="17" t="n">
         <f aca="false">SUMIF($F$11:$F$60,"otvorené",K11:K60)</f>
-        <v>48240.2368744004</v>
+        <v>50396.4575394988</v>
       </c>
       <c r="L62" s="17" t="n">
         <f aca="false">SUMIF($F$11:$F$60,"otvorené",L11:L60)</f>
-        <v>279671.6168744</v>
+        <v>308734.837539499</v>
       </c>
       <c r="M62" s="16"/>
     </row>
@@ -2880,7 +2880,7 @@
       <c r="B67" s="20"/>
       <c r="C67" s="14" t="n">
         <f aca="false">SUMIFS(C$11:C$60,$A$11:$A$60,$A67,$F$11:$F$60,"otvorené")</f>
-        <v>126000</v>
+        <v>152907</v>
       </c>
       <c r="D67" s="20"/>
       <c r="E67" s="20"/>
@@ -2891,11 +2891,11 @@
       <c r="J67" s="20"/>
       <c r="K67" s="14" t="n">
         <f aca="false">SUMIFS(K$11:K$60,$A$11:$A$60,$A67,$F$11:$F$60,"otvorené")</f>
-        <v>28362.1775896885</v>
+        <v>30518.3982547869</v>
       </c>
       <c r="L67" s="15" t="n">
         <f aca="false">SUMIFS(L$11:L$60,$A$11:$A$60,$A67,$F$11:$F$60,"otvorené")</f>
-        <v>154362.177589688</v>
+        <v>183425.398254787</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Daň u Lukáša Cisca: rok 2024, úrok od 30.06.2025
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L5Qg2mKXdzeFPu6vSu8w6V
</commit_message>
<xml_diff>
--- a/supis_dlhov.xlsx
+++ b/supis_dlhov.xlsx
@@ -210,10 +210,10 @@
     <t xml:space="preserve">presný deň neznámy – použitý 31.12.2025, DOPLŇTE</t>
   </si>
   <si>
-    <t xml:space="preserve">Daň za rok 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve">dátum splatnosti neznámy – použitý 31.12.2025, DOPLŇTE</t>
+    <t xml:space="preserve">Daň za rok 2024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jún 2025 podľa zadania, presný deň neznámy – použitý 30.06.2025, DOPLŇTE</t>
   </si>
   <si>
     <t xml:space="preserve">Baláž</t>
@@ -1481,7 +1481,7 @@
         <v>61907</v>
       </c>
       <c r="D22" s="12" t="n">
-        <v>46022</v>
+        <v>45838</v>
       </c>
       <c r="E22" s="10" t="s">
         <v>26</v>
@@ -1491,11 +1491,11 @@
       </c>
       <c r="G22" s="13" t="n">
         <f aca="false">IF(OR($A22="",$D22="",$C22=""),"",MAX(0,$B$3-$D22))</f>
-        <v>284</v>
+        <v>468</v>
       </c>
       <c r="H22" s="13" t="n">
         <f aca="false">IF($G22="","",IF(OR($E22="nie",$B$3&lt;=$D22),0,INT(DATEDIF($D22,$B$3,"m")/$B$5)))</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I22" s="13" t="n">
         <f aca="false">IF($H22="","",IF($E22="nie",0,MAX(0,$B$3-EDATE($D22,$H22*$B$5))))</f>
@@ -1503,15 +1503,15 @@
       </c>
       <c r="J22" s="14" t="n">
         <f aca="false">IF($H22="","",$C22*(1+$B$6)^$H22)</f>
-        <v>66667.067921875</v>
+        <v>70042.0882354199</v>
       </c>
       <c r="K22" s="14" t="n">
         <f aca="false">IF($H22="","",IF($E22="nie",0,$J22*(1+$B$4*$I22/365)-$C22))</f>
-        <v>4960.98237314638</v>
+        <v>8346.1739807869</v>
       </c>
       <c r="L22" s="15" t="n">
         <f aca="false">IF($H22="","",$C22+$K22)</f>
-        <v>66867.9823731464</v>
+        <v>70253.1739807869</v>
       </c>
       <c r="M22" s="10" t="s">
         <v>44</v>
@@ -2810,11 +2810,11 @@
       <c r="J62" s="16"/>
       <c r="K62" s="17" t="n">
         <f aca="false">SUMIF($F$11:$F$60,"otvorené",K11:K60)</f>
-        <v>50396.4575394988</v>
+        <v>53781.6491471393</v>
       </c>
       <c r="L62" s="17" t="n">
         <f aca="false">SUMIF($F$11:$F$60,"otvorené",L11:L60)</f>
-        <v>308734.837539499</v>
+        <v>312120.029147139</v>
       </c>
       <c r="M62" s="16"/>
     </row>
@@ -2891,11 +2891,11 @@
       <c r="J67" s="20"/>
       <c r="K67" s="14" t="n">
         <f aca="false">SUMIFS(K$11:K$60,$A$11:$A$60,$A67,$F$11:$F$60,"otvorené")</f>
-        <v>30518.3982547869</v>
+        <v>33903.5898624274</v>
       </c>
       <c r="L67" s="15" t="n">
         <f aca="false">SUMIFS(L$11:L$60,$A$11:$A$60,$A67,$F$11:$F$60,"otvorené")</f>
-        <v>183425.398254787</v>
+        <v>186810.589862427</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>